<commit_message>
Add kit order list worksheet
</commit_message>
<xml_diff>
--- a/hardware/EnvNode_Parts.xlsx
+++ b/hardware/EnvNode_Parts.xlsx
@@ -8,17 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/Daten/Development/EnvNode/hardware/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A3492C32-62A5-1843-AE61-E7F9447D899E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFC5F107-337F-B94F-A4FC-DE35B5939871}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="20100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="20100" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Parts" sheetId="1" r:id="rId1"/>
     <sheet name="Kits" sheetId="2" r:id="rId2"/>
     <sheet name="Kit_BOM" sheetId="3" r:id="rId3"/>
+    <sheet name="Order_List" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1517" uniqueCount="704">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1586" uniqueCount="720">
   <si>
     <t>Part_ID</t>
   </si>
@@ -2033,6 +2033,9 @@
     <t>hardware/kicad/Modules/FullSize/DuoRelay/DuoRelay.kicad_pcb</t>
   </si>
   <si>
+    <t>Aktueller bestückter KiCad-Umfang plus PCB; DNP-Positionen enthalten und als DNP gekennzeichnet. Mechanische Zusatzteile können anschließend ergänzt werden.</t>
+  </si>
+  <si>
     <t>ENK-00003</t>
   </si>
   <si>
@@ -2045,9 +2048,6 @@
     <t>hardware/kicad/Modules/FullSize/AnalogHydroPressure/AnalogHydroPressure.kicad_pcb</t>
   </si>
   <si>
-    <t>Aktueller bestückter KiCad-Umfang plus PCB; DNP-Positionen enthalten und als DNP gekennzeichnet. Mechanische Zusatzteile können anschließend ergänzt werden.</t>
-  </si>
-  <si>
     <t>Aktueller bestückter KiCad-Umfang einschließlich Busumschaltung plus PCB; DNP-Positionen enthalten und als DNP gekennzeichnet. Mechanische Zusatzteile können anschließend ergänzt werden.</t>
   </si>
   <si>
@@ -2148,6 +2148,54 @@
   </si>
   <si>
     <t>Ergebnis</t>
+  </si>
+  <si>
+    <t>Bestellliste für EnvNode-Bausätze</t>
+  </si>
+  <si>
+    <t>Stückzahlen wählen; die Liste aggregiert gleiche Parts über alle Kits. DNP ist standardmäßig ausgeschlossen.</t>
+  </si>
+  <si>
+    <t>Bausatz</t>
+  </si>
+  <si>
+    <t>Stückzahl</t>
+  </si>
+  <si>
+    <t>Option</t>
+  </si>
+  <si>
+    <t>Auswahl</t>
+  </si>
+  <si>
+    <t>Optional bestellen</t>
+  </si>
+  <si>
+    <t>Nein</t>
+  </si>
+  <si>
+    <t>DNP bestellen</t>
+  </si>
+  <si>
+    <t>Hinweis</t>
+  </si>
+  <si>
+    <t>Bestellmenge wird bei hinterlegter Verpackungseinheit auf das nächste Vielfache aufgerundet.</t>
+  </si>
+  <si>
+    <t>Bedarf</t>
+  </si>
+  <si>
+    <t>Bestellmenge</t>
+  </si>
+  <si>
+    <t>Bestellwert_EUR</t>
+  </si>
+  <si>
+    <t>Import_Status</t>
+  </si>
+  <si>
+    <t>Ja</t>
   </si>
 </sst>
 </file>
@@ -2159,7 +2207,7 @@
     <numFmt numFmtId="165" formatCode="0.00\ &quot;€&quot;"/>
     <numFmt numFmtId="166" formatCode="\€0.00"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -2200,8 +2248,30 @@
       <color rgb="FFFFFFFF"/>
       <name val="Carlito"/>
     </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Carlito"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Carlito"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF375623"/>
+      <name val="Carlito"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF375623"/>
+      <name val="Carlito"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2223,8 +2293,33 @@
         <fgColor rgb="FF1F4E78"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9EAF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF4472C4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE2F0D9"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -2261,13 +2356,124 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFD9E2F3"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFD9E2F3"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD9E2F3"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD9E2F3"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFD9E2F3"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD9E2F3"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFD9E2F3"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFD9E2F3"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD9E2F3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD9E2F3"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD9E2F3"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD9E2F3"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD9E2F3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD9E2F3"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD9E2F3"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FFD9E2F3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD9E2F3"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFD9E2F3"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD9E2F3"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD9E2F3"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD9E2F3"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD9E2F3"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD9E2F3"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FFD9E2F3"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2326,13 +2532,65 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="1" fontId="9" fillId="8" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="9" fillId="8" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="9" fillId="8" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Link" xfId="2" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
     <cellStyle name="Normal" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="10">
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFCE4D6"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF7F6000"/>
@@ -2345,11 +2603,36 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF375623"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFE2F0D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFA6A6A6"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF7F6000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <b/>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
-        <patternFill patternType="solid">
+        <patternFill>
           <bgColor rgb="FFF4CCCC"/>
         </patternFill>
       </fill>
@@ -2408,7 +2691,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="PartsTable" displayName="PartsTable" ref="A1:S77" totalsRowShown="0" dataDxfId="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="PartsTable" displayName="PartsTable" ref="A1:S77" totalsRowShown="0" dataDxfId="9">
   <autoFilter ref="A1:S77" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="19">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Part_ID"/>
@@ -2466,6 +2749,26 @@
     <tableColumn id="11" xr3:uid="{00000000-0010-0000-0200-00000B000000}" name="Unit_Price_EUR"/>
     <tableColumn id="12" xr3:uid="{00000000-0010-0000-0200-00000C000000}" name="Position_Price_EUR"/>
     <tableColumn id="13" xr3:uid="{00000000-0010-0000-0200-00000D000000}" name="Notes"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="OrderListTable" displayName="OrderListTable" ref="A13:K52" totalsRowCount="1">
+  <autoFilter ref="A13:K51" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
+  <tableColumns count="11">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="Part_ID" totalsRowLabel="Ergebnis"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="Description"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="Supplier"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0300-000004000000}" name="Supplier_PN"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0300-000005000000}" name="Bedarf"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0300-000006000000}" name="Packaging_Unit"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0300-000007000000}" name="Bestellmenge"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0300-000008000000}" name="Unit_Price_EUR"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0300-000009000000}" name="Bestellwert_EUR" totalsRowFunction="sum"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0300-00000A000000}" name="Import_Status"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0300-00000B000000}" name="URL" totalsRowFunction="count"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4172,7 +4475,7 @@
         <v>255</v>
       </c>
       <c r="K27" s="6">
-        <v>5.88</v>
+        <v>0.57999999999999996</v>
       </c>
       <c r="L27" s="3" t="s">
         <v>26</v>
@@ -6786,11 +7089,11 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="Q2:Q54">
-    <cfRule type="containsText" dxfId="4" priority="1" operator="containsText" text="Prüfen"/>
-    <cfRule type="containsText" dxfId="3" priority="2" operator="containsText" text="OK"/>
+    <cfRule type="containsText" dxfId="8" priority="1" operator="containsText" text="Prüfen"/>
+    <cfRule type="containsText" dxfId="7" priority="2" operator="containsText" text="OK"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="S2:S54">
-    <cfRule type="duplicateValues" dxfId="2" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="3"/>
   </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation type="list" sqref="Q1:Q1048576" xr:uid="{00000000-0002-0000-0000-000000000000}">
@@ -6886,15 +7189,15 @@
         <v>664</v>
       </c>
       <c r="G3" t="s">
-        <v>669</v>
+        <v>665</v>
       </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="B4" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="C4" t="s">
         <v>656</v>
@@ -6903,10 +7206,10 @@
         <v>657</v>
       </c>
       <c r="E4" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="F4" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="G4" t="s">
         <v>670</v>
@@ -8813,7 +9116,7 @@
     </row>
     <row r="43" spans="1:13">
       <c r="A43" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="B43" t="s">
         <v>656</v>
@@ -8858,7 +9161,7 @@
     </row>
     <row r="44" spans="1:13">
       <c r="A44" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="B44" t="s">
         <v>656</v>
@@ -8903,7 +9206,7 @@
     </row>
     <row r="45" spans="1:13">
       <c r="A45" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="B45" t="s">
         <v>656</v>
@@ -8948,7 +9251,7 @@
     </row>
     <row r="46" spans="1:13">
       <c r="A46" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="B46" t="s">
         <v>656</v>
@@ -8993,7 +9296,7 @@
     </row>
     <row r="47" spans="1:13">
       <c r="A47" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="B47" t="s">
         <v>656</v>
@@ -9038,7 +9341,7 @@
     </row>
     <row r="48" spans="1:13">
       <c r="A48" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="B48" t="s">
         <v>656</v>
@@ -9083,7 +9386,7 @@
     </row>
     <row r="49" spans="1:13">
       <c r="A49" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="B49" t="s">
         <v>656</v>
@@ -9128,7 +9431,7 @@
     </row>
     <row r="50" spans="1:13">
       <c r="A50" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="B50" t="s">
         <v>656</v>
@@ -9173,7 +9476,7 @@
     </row>
     <row r="51" spans="1:13">
       <c r="A51" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="B51" t="s">
         <v>656</v>
@@ -9216,7 +9519,7 @@
     </row>
     <row r="52" spans="1:13">
       <c r="A52" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="B52" t="s">
         <v>656</v>
@@ -9261,7 +9564,7 @@
     </row>
     <row r="53" spans="1:13">
       <c r="A53" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="B53" t="s">
         <v>656</v>
@@ -9304,7 +9607,7 @@
     </row>
     <row r="54" spans="1:13">
       <c r="A54" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="B54" t="s">
         <v>656</v>
@@ -9349,7 +9652,7 @@
     </row>
     <row r="55" spans="1:13">
       <c r="A55" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="B55" t="s">
         <v>656</v>
@@ -9394,7 +9697,7 @@
     </row>
     <row r="56" spans="1:13">
       <c r="A56" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="B56" t="s">
         <v>656</v>
@@ -9439,7 +9742,7 @@
     </row>
     <row r="57" spans="1:13">
       <c r="A57" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="B57" t="s">
         <v>656</v>
@@ -9484,7 +9787,7 @@
     </row>
     <row r="58" spans="1:13">
       <c r="A58" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="B58" t="s">
         <v>656</v>
@@ -9529,7 +9832,7 @@
     </row>
     <row r="59" spans="1:13">
       <c r="A59" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="B59" t="s">
         <v>656</v>
@@ -9574,7 +9877,7 @@
     </row>
     <row r="60" spans="1:13">
       <c r="A60" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="B60" t="s">
         <v>656</v>
@@ -9619,7 +9922,7 @@
     </row>
     <row r="61" spans="1:13">
       <c r="A61" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="B61" t="s">
         <v>656</v>
@@ -9664,7 +9967,7 @@
     </row>
     <row r="62" spans="1:13">
       <c r="A62" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="B62" t="s">
         <v>656</v>
@@ -9710,7 +10013,7 @@
     </row>
     <row r="63" spans="1:13">
       <c r="A63" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="B63" t="s">
         <v>656</v>
@@ -9756,7 +10059,7 @@
     </row>
     <row r="64" spans="1:13">
       <c r="A64" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="B64" t="s">
         <v>656</v>
@@ -9802,7 +10105,7 @@
     </row>
     <row r="65" spans="1:13">
       <c r="A65" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="B65" t="s">
         <v>656</v>
@@ -9859,14 +10162,14 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="G2:G65">
-    <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="DNP"/>
-    <cfRule type="containsText" dxfId="0" priority="2" operator="containsText" text="Optional"/>
+    <cfRule type="containsText" dxfId="5" priority="1" operator="containsText" text="DNP"/>
+    <cfRule type="containsText" dxfId="4" priority="2" operator="containsText" text="Optional"/>
   </conditionalFormatting>
   <dataValidations count="2">
     <dataValidation type="list" sqref="G2:G493 H2:H500" xr:uid="{00000000-0002-0000-0200-000000000000}">
       <formula1>"KiCad,PCB,Mechanical,Cable,Assembly,Consumable"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="G2:G500" xr:uid="{00000000-0002-0000-0200-000002000000}">
+    <dataValidation type="list" sqref="G2:G500" xr:uid="{00000000-0002-0000-0200-000001000000}">
       <formula1>"Bestücken,DNP,Optional"</formula1>
     </dataValidation>
   </dataValidations>
@@ -9874,17 +10177,1926 @@
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
-        <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0200-000001000000}">
-          <x14:formula1>
-            <xm:f>Parts!$A$2:$A$200</xm:f>
-          </x14:formula1>
-          <xm:sqref>E2:E500</xm:sqref>
-        </x14:dataValidation>
-      </x14:dataValidations>
-    </ext>
-  </extLst>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <dimension ref="A1:K52"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="13" customWidth="1"/>
+    <col min="2" max="2" width="35" customWidth="1"/>
+    <col min="3" max="3" width="15" customWidth="1"/>
+    <col min="4" max="4" width="22" customWidth="1"/>
+    <col min="5" max="5" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15" customWidth="1"/>
+    <col min="7" max="8" width="14" customWidth="1"/>
+    <col min="9" max="9" width="15" customWidth="1"/>
+    <col min="10" max="10" width="20" customWidth="1"/>
+    <col min="11" max="11" width="255.83203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" ht="30" customHeight="1">
+      <c r="A1" s="40" t="s">
+        <v>704</v>
+      </c>
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="40"/>
+      <c r="I1" s="40"/>
+      <c r="J1" s="40"/>
+      <c r="K1" s="40"/>
+    </row>
+    <row r="2" spans="1:11" ht="26" customHeight="1">
+      <c r="A2" s="41" t="s">
+        <v>705</v>
+      </c>
+      <c r="B2" s="41"/>
+      <c r="C2" s="41"/>
+      <c r="D2" s="41"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="41"/>
+      <c r="G2" s="41"/>
+      <c r="H2" s="41"/>
+      <c r="I2" s="41"/>
+      <c r="J2" s="41"/>
+      <c r="K2" s="41"/>
+    </row>
+    <row r="4" spans="1:11">
+      <c r="A4" s="24" t="s">
+        <v>648</v>
+      </c>
+      <c r="B4" s="24" t="s">
+        <v>706</v>
+      </c>
+      <c r="C4" s="24" t="s">
+        <v>707</v>
+      </c>
+      <c r="E4" s="24" t="s">
+        <v>708</v>
+      </c>
+      <c r="F4" s="24" t="s">
+        <v>709</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11">
+      <c r="A5" s="25" t="s">
+        <v>654</v>
+      </c>
+      <c r="B5" s="26" t="s">
+        <v>655</v>
+      </c>
+      <c r="C5" s="31">
+        <v>1</v>
+      </c>
+      <c r="E5" s="25" t="s">
+        <v>710</v>
+      </c>
+      <c r="F5" s="34" t="s">
+        <v>711</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11">
+      <c r="A6" s="27" t="s">
+        <v>661</v>
+      </c>
+      <c r="B6" s="28" t="s">
+        <v>662</v>
+      </c>
+      <c r="C6" s="32">
+        <v>2</v>
+      </c>
+      <c r="E6" s="29" t="s">
+        <v>712</v>
+      </c>
+      <c r="F6" s="35" t="s">
+        <v>719</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11">
+      <c r="A7" s="29" t="s">
+        <v>666</v>
+      </c>
+      <c r="B7" s="30" t="s">
+        <v>667</v>
+      </c>
+      <c r="C7" s="33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="16">
+      <c r="E8" s="37" t="s">
+        <v>713</v>
+      </c>
+      <c r="F8" s="42" t="s">
+        <v>714</v>
+      </c>
+      <c r="G8" s="42"/>
+      <c r="H8" s="42"/>
+      <c r="I8" s="42"/>
+      <c r="J8" s="42"/>
+      <c r="K8" s="42"/>
+    </row>
+    <row r="9" spans="1:11">
+      <c r="E9" s="36"/>
+      <c r="F9" s="42"/>
+      <c r="G9" s="42"/>
+      <c r="H9" s="42"/>
+      <c r="I9" s="42"/>
+      <c r="J9" s="42"/>
+      <c r="K9" s="42"/>
+    </row>
+    <row r="13" spans="1:11" ht="15" customHeight="1">
+      <c r="A13" t="s">
+        <v>0</v>
+      </c>
+      <c r="B13" t="s">
+        <v>2</v>
+      </c>
+      <c r="C13" t="s">
+        <v>7</v>
+      </c>
+      <c r="D13" t="s">
+        <v>8</v>
+      </c>
+      <c r="E13" t="s">
+        <v>715</v>
+      </c>
+      <c r="F13" t="s">
+        <v>12</v>
+      </c>
+      <c r="G13" t="s">
+        <v>716</v>
+      </c>
+      <c r="H13" t="s">
+        <v>10</v>
+      </c>
+      <c r="I13" t="s">
+        <v>717</v>
+      </c>
+      <c r="J13" t="s">
+        <v>718</v>
+      </c>
+      <c r="K13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="15" customHeight="1">
+      <c r="A14" t="s">
+        <v>58</v>
+      </c>
+      <c r="B14" s="39" t="str">
+        <f>IFERROR(VLOOKUP($A14,Parts!$A$2:$S$200,3,FALSE),"")</f>
+        <v>4.7 kOhm 1% SMD 1206</v>
+      </c>
+      <c r="C14" t="str">
+        <f>IFERROR(VLOOKUP($A14,Parts!$A$2:$S$200,8,FALSE),"")</f>
+        <v>reichelt</v>
+      </c>
+      <c r="D14" t="str">
+        <f>IFERROR(VLOOKUP($A14,Parts!$A$2:$S$200,9,FALSE),"")</f>
+        <v>VIS CRCW12064K7</v>
+      </c>
+      <c r="E14" s="21">
+        <f>SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A14,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$5+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A14,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Optional")*$C$5,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A14,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"DNP")*$C$5,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A14,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$6+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A14,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Optional")*$C$6,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A14,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"DNP")*$C$6,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A14,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$7+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A14,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Optional")*$C$7,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A14,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"DNP")*$C$7,0)</f>
+        <v>4</v>
+      </c>
+      <c r="F14" s="21">
+        <f>IFERROR(VLOOKUP($A14,Parts!$A$2:$S$200,13,FALSE),"")</f>
+        <v>0</v>
+      </c>
+      <c r="G14" s="21">
+        <f t="shared" ref="G14:G51" si="0">IF($E14=0,0,IF(OR($F14="",$F14=0),$E14,CEILING($E14,$F14)))</f>
+        <v>4</v>
+      </c>
+      <c r="H14" s="38">
+        <f>IFERROR(VLOOKUP($A14,Parts!$A$2:$S$200,11,FALSE),0)</f>
+        <v>0.15</v>
+      </c>
+      <c r="I14" s="38">
+        <f t="shared" ref="I14:I51" si="1">$G14*$H14</f>
+        <v>0.6</v>
+      </c>
+      <c r="J14" t="str">
+        <f t="shared" ref="J14:J51" si="2">IF($E14=0,"Nicht benötigt",IF(LOWER($C14)&lt;&gt;"reichelt","Anderer Lieferant",IF($D14="","Supplier-PN fehlt","Reichelt bereit")))</f>
+        <v>Reichelt bereit</v>
+      </c>
+      <c r="K14" t="str">
+        <f>IFERROR(VLOOKUP($A14,Parts!$A$2:$S$200,10,FALSE),"")</f>
+        <v>https://www.reichelt.de/de/de/shop/produkt/smd-widerstand_1206_4_7_kohm_250_mw_1_-238119</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="15" customHeight="1">
+      <c r="A15" t="s">
+        <v>70</v>
+      </c>
+      <c r="B15" s="39" t="str">
+        <f>IFERROR(VLOOKUP($A15,Parts!$A$2:$S$200,3,FALSE),"")</f>
+        <v>100 nF Keramik SMD</v>
+      </c>
+      <c r="C15" t="str">
+        <f>IFERROR(VLOOKUP($A15,Parts!$A$2:$S$200,8,FALSE),"")</f>
+        <v>reichelt</v>
+      </c>
+      <c r="D15" t="str">
+        <f>IFERROR(VLOOKUP($A15,Parts!$A$2:$S$200,9,FALSE),"")</f>
+        <v>KEM X7R1206A100N</v>
+      </c>
+      <c r="E15" s="21">
+        <f>SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A15,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$5+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A15,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Optional")*$C$5,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A15,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"DNP")*$C$5,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A15,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$6+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A15,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Optional")*$C$6,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A15,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"DNP")*$C$6,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A15,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$7+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A15,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Optional")*$C$7,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A15,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"DNP")*$C$7,0)</f>
+        <v>5</v>
+      </c>
+      <c r="F15" s="21">
+        <f>IFERROR(VLOOKUP($A15,Parts!$A$2:$S$200,13,FALSE),"")</f>
+        <v>10</v>
+      </c>
+      <c r="G15" s="21">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="H15" s="38">
+        <f>IFERROR(VLOOKUP($A15,Parts!$A$2:$S$200,11,FALSE),0)</f>
+        <v>0.24</v>
+      </c>
+      <c r="I15" s="38">
+        <f t="shared" si="1"/>
+        <v>2.4</v>
+      </c>
+      <c r="J15" t="str">
+        <f t="shared" si="2"/>
+        <v>Reichelt bereit</v>
+      </c>
+      <c r="K15" t="str">
+        <f>IFERROR(VLOOKUP($A15,Parts!$A$2:$S$200,10,FALSE),"")</f>
+        <v>https://www.reichelt.de/de/de/shop/produkt/vielschicht_kerko_1206_100_nf_10_x7r_100_v_125_c-207151</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" ht="15" customHeight="1">
+      <c r="A16" t="s">
+        <v>82</v>
+      </c>
+      <c r="B16" s="39" t="str">
+        <f>IFERROR(VLOOKUP($A16,Parts!$A$2:$S$200,3,FALSE),"")</f>
+        <v>10 uF Keramik SMD</v>
+      </c>
+      <c r="C16" t="str">
+        <f>IFERROR(VLOOKUP($A16,Parts!$A$2:$S$200,8,FALSE),"")</f>
+        <v>reichelt</v>
+      </c>
+      <c r="D16" t="str">
+        <f>IFERROR(VLOOKUP($A16,Parts!$A$2:$S$200,9,FALSE),"")</f>
+        <v>12063C106KAT2A</v>
+      </c>
+      <c r="E16" s="21">
+        <f>SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A16,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$5+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A16,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Optional")*$C$5,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A16,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"DNP")*$C$5,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A16,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$6+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A16,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Optional")*$C$6,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A16,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"DNP")*$C$6,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A16,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$7+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A16,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Optional")*$C$7,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A16,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"DNP")*$C$7,0)</f>
+        <v>1</v>
+      </c>
+      <c r="F16" s="21">
+        <f>IFERROR(VLOOKUP($A16,Parts!$A$2:$S$200,13,FALSE),"")</f>
+        <v>10</v>
+      </c>
+      <c r="G16" s="21">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="H16" s="38">
+        <f>IFERROR(VLOOKUP($A16,Parts!$A$2:$S$200,11,FALSE),0)</f>
+        <v>0.11</v>
+      </c>
+      <c r="I16" s="38">
+        <f t="shared" si="1"/>
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="J16" t="str">
+        <f t="shared" si="2"/>
+        <v>Reichelt bereit</v>
+      </c>
+      <c r="K16" t="str">
+        <f>IFERROR(VLOOKUP($A16,Parts!$A$2:$S$200,10,FALSE),"")</f>
+        <v>https://www.reichelt.de/de/de/shop/produkt/mlcc_1206_10_f_25_v_-10_x7r-409262</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="15" customHeight="1">
+      <c r="A17" t="s">
+        <v>91</v>
+      </c>
+      <c r="B17" s="39" t="str">
+        <f>IFERROR(VLOOKUP($A17,Parts!$A$2:$S$200,3,FALSE),"")</f>
+        <v>47 uF 10V Tantal</v>
+      </c>
+      <c r="C17" t="str">
+        <f>IFERROR(VLOOKUP($A17,Parts!$A$2:$S$200,8,FALSE),"")</f>
+        <v>reichelt</v>
+      </c>
+      <c r="D17" t="str">
+        <f>IFERROR(VLOOKUP($A17,Parts!$A$2:$S$200,9,FALSE),"")</f>
+        <v>TAJ 3528 47/10</v>
+      </c>
+      <c r="E17" s="21">
+        <f>SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A17,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$5+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A17,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Optional")*$C$5,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A17,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"DNP")*$C$5,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A17,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$6+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A17,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Optional")*$C$6,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A17,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"DNP")*$C$6,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A17,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$7+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A17,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Optional")*$C$7,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A17,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"DNP")*$C$7,0)</f>
+        <v>1</v>
+      </c>
+      <c r="F17" s="21">
+        <f>IFERROR(VLOOKUP($A17,Parts!$A$2:$S$200,13,FALSE),"")</f>
+        <v>0</v>
+      </c>
+      <c r="G17" s="21">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="H17" s="38">
+        <f>IFERROR(VLOOKUP($A17,Parts!$A$2:$S$200,11,FALSE),0)</f>
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="I17" s="38">
+        <f t="shared" si="1"/>
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="J17" t="str">
+        <f t="shared" si="2"/>
+        <v>Reichelt bereit</v>
+      </c>
+      <c r="K17" t="str">
+        <f>IFERROR(VLOOKUP($A17,Parts!$A$2:$S$200,10,FALSE),"")</f>
+        <v>https://www.reichelt.de/de/de/shop/produkt/smd-tantal_kondensator_47_f_10_v-167014</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" ht="15" customHeight="1">
+      <c r="A18" t="s">
+        <v>100</v>
+      </c>
+      <c r="B18" s="39" t="str">
+        <f>IFERROR(VLOOKUP($A18,Parts!$A$2:$S$200,3,FALSE),"")</f>
+        <v>LDO 3.3V SOT-223</v>
+      </c>
+      <c r="C18" t="str">
+        <f>IFERROR(VLOOKUP($A18,Parts!$A$2:$S$200,8,FALSE),"")</f>
+        <v>reichelt</v>
+      </c>
+      <c r="D18" t="str">
+        <f>IFERROR(VLOOKUP($A18,Parts!$A$2:$S$200,9,FALSE),"")</f>
+        <v>LM 3940 IMP-3</v>
+      </c>
+      <c r="E18" s="21">
+        <f>SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A18,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$5+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A18,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Optional")*$C$5,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A18,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"DNP")*$C$5,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A18,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$6+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A18,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Optional")*$C$6,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A18,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"DNP")*$C$6,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A18,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$7+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A18,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Optional")*$C$7,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A18,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"DNP")*$C$7,0)</f>
+        <v>1</v>
+      </c>
+      <c r="F18" s="21">
+        <f>IFERROR(VLOOKUP($A18,Parts!$A$2:$S$200,13,FALSE),"")</f>
+        <v>3</v>
+      </c>
+      <c r="G18" s="21">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="H18" s="38">
+        <f>IFERROR(VLOOKUP($A18,Parts!$A$2:$S$200,11,FALSE),0)</f>
+        <v>1</v>
+      </c>
+      <c r="I18" s="38">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="J18" t="str">
+        <f t="shared" si="2"/>
+        <v>Reichelt bereit</v>
+      </c>
+      <c r="K18" t="str">
+        <f>IFERROR(VLOOKUP($A18,Parts!$A$2:$S$200,10,FALSE),"")</f>
+        <v>https://www.reichelt.de/de/de/shop/produkt/ldo-spannungsregler_fix_3_3_vout_1_a_sot-223-109407?search=LM3940%2520&amp;</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" ht="15" customHeight="1">
+      <c r="A19" t="s">
+        <v>111</v>
+      </c>
+      <c r="B19" s="39" t="str">
+        <f>IFERROR(VLOOKUP($A19,Parts!$A$2:$S$200,3,FALSE),"")</f>
+        <v>ESP32-DevKitC</v>
+      </c>
+      <c r="C19">
+        <f>IFERROR(VLOOKUP($A19,Parts!$A$2:$S$200,8,FALSE),"")</f>
+        <v>0</v>
+      </c>
+      <c r="D19">
+        <f>IFERROR(VLOOKUP($A19,Parts!$A$2:$S$200,9,FALSE),"")</f>
+        <v>0</v>
+      </c>
+      <c r="E19" s="21">
+        <f>SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A19,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$5+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A19,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Optional")*$C$5,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A19,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"DNP")*$C$5,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A19,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$6+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A19,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Optional")*$C$6,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A19,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"DNP")*$C$6,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A19,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$7+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A19,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Optional")*$C$7,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A19,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"DNP")*$C$7,0)</f>
+        <v>1</v>
+      </c>
+      <c r="F19" s="21">
+        <f>IFERROR(VLOOKUP($A19,Parts!$A$2:$S$200,13,FALSE),"")</f>
+        <v>3</v>
+      </c>
+      <c r="G19" s="21">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="H19" s="38">
+        <f>IFERROR(VLOOKUP($A19,Parts!$A$2:$S$200,11,FALSE),0)</f>
+        <v>5</v>
+      </c>
+      <c r="I19" s="38">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="J19" t="str">
+        <f t="shared" si="2"/>
+        <v>Anderer Lieferant</v>
+      </c>
+      <c r="K19">
+        <f>IFERROR(VLOOKUP($A19,Parts!$A$2:$S$200,10,FALSE),"")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="15" customHeight="1">
+      <c r="A20" t="s">
+        <v>126</v>
+      </c>
+      <c r="B20" s="39" t="str">
+        <f>IFERROR(VLOOKUP($A20,Parts!$A$2:$S$200,3,FALSE),"")</f>
+        <v>JST - Stiftleiste, gerade, 1x2-polig - PH</v>
+      </c>
+      <c r="C20" t="str">
+        <f>IFERROR(VLOOKUP($A20,Parts!$A$2:$S$200,8,FALSE),"")</f>
+        <v>reichelt</v>
+      </c>
+      <c r="D20" t="str">
+        <f>IFERROR(VLOOKUP($A20,Parts!$A$2:$S$200,9,FALSE),"")</f>
+        <v>JST PH2P ST</v>
+      </c>
+      <c r="E20" s="21">
+        <f>SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A20,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$5+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A20,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Optional")*$C$5,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A20,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"DNP")*$C$5,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A20,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$6+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A20,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Optional")*$C$6,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A20,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"DNP")*$C$6,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A20,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$7+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A20,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Optional")*$C$7,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A20,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"DNP")*$C$7,0)</f>
+        <v>1</v>
+      </c>
+      <c r="F20" s="21">
+        <f>IFERROR(VLOOKUP($A20,Parts!$A$2:$S$200,13,FALSE),"")</f>
+        <v>0</v>
+      </c>
+      <c r="G20" s="21">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="H20" s="38">
+        <f>IFERROR(VLOOKUP($A20,Parts!$A$2:$S$200,11,FALSE),0)</f>
+        <v>1.3</v>
+      </c>
+      <c r="I20" s="38">
+        <f t="shared" si="1"/>
+        <v>1.3</v>
+      </c>
+      <c r="J20" t="str">
+        <f t="shared" si="2"/>
+        <v>Reichelt bereit</v>
+      </c>
+      <c r="K20" t="str">
+        <f>IFERROR(VLOOKUP($A20,Parts!$A$2:$S$200,10,FALSE),"")</f>
+        <v>https://www.reichelt.de/de/de/shop/produkt/jst_-_stiftleiste_gerade_1x2-polig_-_ph-185049</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="26.25" customHeight="1">
+      <c r="A21" t="s">
+        <v>158</v>
+      </c>
+      <c r="B21" s="39" t="str">
+        <f>IFERROR(VLOOKUP($A21,Parts!$A$2:$S$200,3,FALSE),"")</f>
+        <v>SMD-Widerstand, 1206, 100 kOhm, 250 mW, 0,1%</v>
+      </c>
+      <c r="C21" t="str">
+        <f>IFERROR(VLOOKUP($A21,Parts!$A$2:$S$200,8,FALSE),"")</f>
+        <v>reichelt</v>
+      </c>
+      <c r="D21" t="str">
+        <f>IFERROR(VLOOKUP($A21,Parts!$A$2:$S$200,9,FALSE),"")</f>
+        <v>PAN ERA8AEB104V</v>
+      </c>
+      <c r="E21" s="21">
+        <f>SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A21,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$5+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A21,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Optional")*$C$5,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A21,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"DNP")*$C$5,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A21,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$6+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A21,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Optional")*$C$6,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A21,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"DNP")*$C$6,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A21,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$7+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A21,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Optional")*$C$7,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A21,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"DNP")*$C$7,0)</f>
+        <v>4</v>
+      </c>
+      <c r="F21" s="21">
+        <f>IFERROR(VLOOKUP($A21,Parts!$A$2:$S$200,13,FALSE),"")</f>
+        <v>0</v>
+      </c>
+      <c r="G21" s="21">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="H21" s="38">
+        <f>IFERROR(VLOOKUP($A21,Parts!$A$2:$S$200,11,FALSE),0)</f>
+        <v>0.83</v>
+      </c>
+      <c r="I21" s="38">
+        <f t="shared" si="1"/>
+        <v>3.32</v>
+      </c>
+      <c r="J21" t="str">
+        <f t="shared" si="2"/>
+        <v>Reichelt bereit</v>
+      </c>
+      <c r="K21" t="str">
+        <f>IFERROR(VLOOKUP($A21,Parts!$A$2:$S$200,10,FALSE),"")</f>
+        <v>https://www.reichelt.de/de/de/shop/produkt/smd-widerstand_1206_100_kohm_250_mw_0_1_-238081</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" ht="15" customHeight="1">
+      <c r="A22" t="s">
+        <v>217</v>
+      </c>
+      <c r="B22" s="39" t="str">
+        <f>IFERROR(VLOOKUP($A22,Parts!$A$2:$S$200,3,FALSE),"")</f>
+        <v>Steck-Printrelais, 1 CO, 6 A, 5 V DC sensitiv</v>
+      </c>
+      <c r="C22" t="str">
+        <f>IFERROR(VLOOKUP($A22,Parts!$A$2:$S$200,8,FALSE),"")</f>
+        <v>reichelt</v>
+      </c>
+      <c r="D22" t="str">
+        <f>IFERROR(VLOOKUP($A22,Parts!$A$2:$S$200,9,FALSE),"")</f>
+        <v>FIN 34.51.7 5V</v>
+      </c>
+      <c r="E22" s="21">
+        <f>SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A22,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$5+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A22,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Optional")*$C$5,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A22,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"DNP")*$C$5,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A22,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$6+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A22,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Optional")*$C$6,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A22,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"DNP")*$C$6,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A22,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$7+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A22,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Optional")*$C$7,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A22,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"DNP")*$C$7,0)</f>
+        <v>4</v>
+      </c>
+      <c r="F22" s="21">
+        <f>IFERROR(VLOOKUP($A22,Parts!$A$2:$S$200,13,FALSE),"")</f>
+        <v>0</v>
+      </c>
+      <c r="G22" s="21">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="H22" s="38">
+        <f>IFERROR(VLOOKUP($A22,Parts!$A$2:$S$200,11,FALSE),0)</f>
+        <v>5.8</v>
+      </c>
+      <c r="I22" s="38">
+        <f t="shared" si="1"/>
+        <v>23.2</v>
+      </c>
+      <c r="J22" t="str">
+        <f t="shared" si="2"/>
+        <v>Reichelt bereit</v>
+      </c>
+      <c r="K22" t="str">
+        <f>IFERROR(VLOOKUP($A22,Parts!$A$2:$S$200,10,FALSE),"")</f>
+        <v>https://www.reichelt.de/de/de/shop/produkt/steck-printrelais_1_co_6_a_5_v_dc_sensitiv-259179?PROVID=2788&amp;gad_source=1&amp;gad_campaignid=21154720511&amp;gbraid=0AAAAADwnxtb50MtqKwtKae8MAeGQARqWX&amp;gclid=CjwKCAjw7p_UBhBlEiwAhpIs72D6cK8XQyuxcrvb0uftoYY3618BT3lTyYSWWSou1J99G9udBcpsbhoCJbcQAvD_BwE</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" ht="26.25" customHeight="1">
+      <c r="A23" t="s">
+        <v>228</v>
+      </c>
+      <c r="B23" s="39" t="str">
+        <f>IFERROR(VLOOKUP($A23,Parts!$A$2:$S$200,3,FALSE),"")</f>
+        <v>I²C-EEPROM 2 Kbit mit vorprogrammierter EUI-64 und zwei Adresspins</v>
+      </c>
+      <c r="C23">
+        <f>IFERROR(VLOOKUP($A23,Parts!$A$2:$S$200,8,FALSE),"")</f>
+        <v>0</v>
+      </c>
+      <c r="D23">
+        <f>IFERROR(VLOOKUP($A23,Parts!$A$2:$S$200,9,FALSE),"")</f>
+        <v>0</v>
+      </c>
+      <c r="E23" s="21">
+        <f>SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A23,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$5+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A23,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Optional")*$C$5,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A23,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"DNP")*$C$5,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A23,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$6+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A23,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Optional")*$C$6,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A23,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"DNP")*$C$6,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A23,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$7+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A23,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Optional")*$C$7,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A23,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"DNP")*$C$7,0)</f>
+        <v>3</v>
+      </c>
+      <c r="F23" s="21">
+        <f>IFERROR(VLOOKUP($A23,Parts!$A$2:$S$200,13,FALSE),"")</f>
+        <v>0</v>
+      </c>
+      <c r="G23" s="21">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="H23" s="38">
+        <f>IFERROR(VLOOKUP($A23,Parts!$A$2:$S$200,11,FALSE),0)</f>
+        <v>0</v>
+      </c>
+      <c r="I23" s="38">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J23" t="str">
+        <f t="shared" si="2"/>
+        <v>Anderer Lieferant</v>
+      </c>
+      <c r="K23">
+        <f>IFERROR(VLOOKUP($A23,Parts!$A$2:$S$200,10,FALSE),"")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" ht="15" customHeight="1">
+      <c r="A24" t="s">
+        <v>248</v>
+      </c>
+      <c r="B24" s="39" t="str">
+        <f>IFERROR(VLOOKUP($A24,Parts!$A$2:$S$200,3,FALSE),"")</f>
+        <v>JST-SH Stiftleiste, 4-polig, horizontal</v>
+      </c>
+      <c r="C24" t="str">
+        <f>IFERROR(VLOOKUP($A24,Parts!$A$2:$S$200,8,FALSE),"")</f>
+        <v>rs-online</v>
+      </c>
+      <c r="D24" t="str">
+        <f>IFERROR(VLOOKUP($A24,Parts!$A$2:$S$200,9,FALSE),"")</f>
+        <v>515-1513</v>
+      </c>
+      <c r="E24" s="21">
+        <f>SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A24,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$5+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A24,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Optional")*$C$5,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A24,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"DNP")*$C$5,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A24,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$6+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A24,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Optional")*$C$6,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A24,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"DNP")*$C$6,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A24,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$7+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A24,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Optional")*$C$7,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A24,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"DNP")*$C$7,0)</f>
+        <v>2</v>
+      </c>
+      <c r="F24" s="21">
+        <f>IFERROR(VLOOKUP($A24,Parts!$A$2:$S$200,13,FALSE),"")</f>
+        <v>10</v>
+      </c>
+      <c r="G24" s="21">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="H24" s="38">
+        <f>IFERROR(VLOOKUP($A24,Parts!$A$2:$S$200,11,FALSE),0)</f>
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="I24" s="38">
+        <f t="shared" si="1"/>
+        <v>5.8</v>
+      </c>
+      <c r="J24" t="str">
+        <f t="shared" si="2"/>
+        <v>Anderer Lieferant</v>
+      </c>
+      <c r="K24" t="str">
+        <f>IFERROR(VLOOKUP($A24,Parts!$A$2:$S$200,10,FALSE),"")</f>
+        <v>https://de.rs-online.com/web/p/leiterplatten-header/5151513?cm_mmc=DE-PLA-DS3A-_-google-_-CSS_DE_DE_PMAX_Catch+All-_--_-5151513&amp;matchtype=&amp;&amp;gclsrc=aw.ds&amp;gad_source=1&amp;gad_campaignid=20579356490&amp;gbraid=0AAAAADkeWNMTclazDyI9zcjcIGwAjXoW9&amp;gclid=Cj0KCQjwnbrUBhDOARIsAKKhPpdLcMySAoEWll9Yd6dc_BCjxUsLFQOO7peTYM0DUy9ctvB7N_5s3bUaAoLZEALw_wcB</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" ht="15" customHeight="1">
+      <c r="A25" t="s">
+        <v>259</v>
+      </c>
+      <c r="B25" s="39" t="str">
+        <f>IFERROR(VLOOKUP($A25,Parts!$A$2:$S$200,3,FALSE),"")</f>
+        <v>16-Bit ADC mit I²C</v>
+      </c>
+      <c r="C25">
+        <f>IFERROR(VLOOKUP($A25,Parts!$A$2:$S$200,8,FALSE),"")</f>
+        <v>0</v>
+      </c>
+      <c r="D25">
+        <f>IFERROR(VLOOKUP($A25,Parts!$A$2:$S$200,9,FALSE),"")</f>
+        <v>0</v>
+      </c>
+      <c r="E25" s="21">
+        <f>SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A25,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$5+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A25,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Optional")*$C$5,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A25,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"DNP")*$C$5,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A25,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$6+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A25,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Optional")*$C$6,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A25,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"DNP")*$C$6,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A25,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$7+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A25,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Optional")*$C$7,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A25,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"DNP")*$C$7,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F25" s="21">
+        <f>IFERROR(VLOOKUP($A25,Parts!$A$2:$S$200,13,FALSE),"")</f>
+        <v>0</v>
+      </c>
+      <c r="G25" s="21">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H25" s="38">
+        <f>IFERROR(VLOOKUP($A25,Parts!$A$2:$S$200,11,FALSE),0)</f>
+        <v>0</v>
+      </c>
+      <c r="I25" s="38">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J25" t="str">
+        <f t="shared" si="2"/>
+        <v>Nicht benötigt</v>
+      </c>
+      <c r="K25">
+        <f>IFERROR(VLOOKUP($A25,Parts!$A$2:$S$200,10,FALSE),"")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" ht="15" customHeight="1">
+      <c r="A26" t="s">
+        <v>266</v>
+      </c>
+      <c r="B26" s="39" t="str">
+        <f>IFERROR(VLOOKUP($A26,Parts!$A$2:$S$200,3,FALSE),"")</f>
+        <v>Keramikkondensator 1 µF SMD</v>
+      </c>
+      <c r="C26" t="str">
+        <f>IFERROR(VLOOKUP($A26,Parts!$A$2:$S$200,8,FALSE),"")</f>
+        <v>reichelt</v>
+      </c>
+      <c r="D26" t="str">
+        <f>IFERROR(VLOOKUP($A26,Parts!$A$2:$S$200,9,FALSE),"")</f>
+        <v>12065C105JAT2A</v>
+      </c>
+      <c r="E26" s="21">
+        <f>SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A26,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$5+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A26,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Optional")*$C$5,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A26,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"DNP")*$C$5,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A26,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$6+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A26,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Optional")*$C$6,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A26,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"DNP")*$C$6,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A26,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$7+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A26,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Optional")*$C$7,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A26,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"DNP")*$C$7,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F26" s="21">
+        <f>IFERROR(VLOOKUP($A26,Parts!$A$2:$S$200,13,FALSE),"")</f>
+        <v>0</v>
+      </c>
+      <c r="G26" s="21">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H26" s="38">
+        <f>IFERROR(VLOOKUP($A26,Parts!$A$2:$S$200,11,FALSE),0)</f>
+        <v>0.16</v>
+      </c>
+      <c r="I26" s="38">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J26" t="str">
+        <f t="shared" si="2"/>
+        <v>Nicht benötigt</v>
+      </c>
+      <c r="K26" t="str">
+        <f>IFERROR(VLOOKUP($A26,Parts!$A$2:$S$200,10,FALSE),"")</f>
+        <v>https://www.reichelt.de/de/de/shop/produkt/mlcc_1206_1_f_50_v_-5_x7r-409277</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" ht="15" customHeight="1">
+      <c r="A27" t="s">
+        <v>273</v>
+      </c>
+      <c r="B27" s="39" t="str">
+        <f>IFERROR(VLOOKUP($A27,Parts!$A$2:$S$200,3,FALSE),"")</f>
+        <v>Dual-Schottky-Diode BAT54S</v>
+      </c>
+      <c r="C27" t="str">
+        <f>IFERROR(VLOOKUP($A27,Parts!$A$2:$S$200,8,FALSE),"")</f>
+        <v>reichelt</v>
+      </c>
+      <c r="D27" t="str">
+        <f>IFERROR(VLOOKUP($A27,Parts!$A$2:$S$200,9,FALSE),"")</f>
+        <v>BAT 54S DIO</v>
+      </c>
+      <c r="E27" s="21">
+        <f>SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A27,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$5+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A27,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Optional")*$C$5,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A27,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"DNP")*$C$5,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A27,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$6+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A27,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Optional")*$C$6,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A27,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"DNP")*$C$6,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A27,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$7+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A27,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Optional")*$C$7,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A27,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"DNP")*$C$7,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F27" s="21">
+        <f>IFERROR(VLOOKUP($A27,Parts!$A$2:$S$200,13,FALSE),"")</f>
+        <v>0</v>
+      </c>
+      <c r="G27" s="21">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H27" s="38">
+        <f>IFERROR(VLOOKUP($A27,Parts!$A$2:$S$200,11,FALSE),0)</f>
+        <v>0.04</v>
+      </c>
+      <c r="I27" s="38">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J27" t="str">
+        <f t="shared" si="2"/>
+        <v>Nicht benötigt</v>
+      </c>
+      <c r="K27" t="str">
+        <f>IFERROR(VLOOKUP($A27,Parts!$A$2:$S$200,10,FALSE),"")</f>
+        <v>https://www.reichelt.de/de/de/shop/produkt/schottkydiode_30_v_0_2_a_sot-23-219176</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" ht="15" customHeight="1">
+      <c r="A28" t="s">
+        <v>290</v>
+      </c>
+      <c r="B28" s="39" t="str">
+        <f>IFERROR(VLOOKUP($A28,Parts!$A$2:$S$200,3,FALSE),"")</f>
+        <v>Buchsenleiste 1x2, vertikal</v>
+      </c>
+      <c r="C28">
+        <f>IFERROR(VLOOKUP($A28,Parts!$A$2:$S$200,8,FALSE),"")</f>
+        <v>0</v>
+      </c>
+      <c r="D28">
+        <f>IFERROR(VLOOKUP($A28,Parts!$A$2:$S$200,9,FALSE),"")</f>
+        <v>0</v>
+      </c>
+      <c r="E28" s="21">
+        <f>SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A28,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$5+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A28,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Optional")*$C$5,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A28,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"DNP")*$C$5,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A28,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$6+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A28,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Optional")*$C$6,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A28,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"DNP")*$C$6,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A28,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$7+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A28,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Optional")*$C$7,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A28,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"DNP")*$C$7,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F28" s="21">
+        <f>IFERROR(VLOOKUP($A28,Parts!$A$2:$S$200,13,FALSE),"")</f>
+        <v>0</v>
+      </c>
+      <c r="G28" s="21">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H28" s="38">
+        <f>IFERROR(VLOOKUP($A28,Parts!$A$2:$S$200,11,FALSE),0)</f>
+        <v>0</v>
+      </c>
+      <c r="I28" s="38">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J28" t="str">
+        <f t="shared" si="2"/>
+        <v>Nicht benötigt</v>
+      </c>
+      <c r="K28">
+        <f>IFERROR(VLOOKUP($A28,Parts!$A$2:$S$200,10,FALSE),"")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" ht="26.25" customHeight="1">
+      <c r="A29" t="s">
+        <v>295</v>
+      </c>
+      <c r="B29" s="39" t="str">
+        <f>IFERROR(VLOOKUP($A29,Parts!$A$2:$S$200,3,FALSE),"")</f>
+        <v>Widerstand, Metallschicht, 150 Ohm, 0207, 250 mW, 0,1%</v>
+      </c>
+      <c r="C29" t="str">
+        <f>IFERROR(VLOOKUP($A29,Parts!$A$2:$S$200,8,FALSE),"")</f>
+        <v>reichelt</v>
+      </c>
+      <c r="D29" t="str">
+        <f>IFERROR(VLOOKUP($A29,Parts!$A$2:$S$200,9,FALSE),"")</f>
+        <v>ARC MRA0207 150R</v>
+      </c>
+      <c r="E29" s="21">
+        <f>SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A29,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$5+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A29,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Optional")*$C$5,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A29,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"DNP")*$C$5,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A29,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$6+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A29,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Optional")*$C$6,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A29,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"DNP")*$C$6,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A29,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$7+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A29,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Optional")*$C$7,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A29,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"DNP")*$C$7,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F29" s="21">
+        <f>IFERROR(VLOOKUP($A29,Parts!$A$2:$S$200,13,FALSE),"")</f>
+        <v>0</v>
+      </c>
+      <c r="G29" s="21">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H29" s="38">
+        <f>IFERROR(VLOOKUP($A29,Parts!$A$2:$S$200,11,FALSE),0)</f>
+        <v>1.3</v>
+      </c>
+      <c r="I29" s="38">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J29" t="str">
+        <f t="shared" si="2"/>
+        <v>Nicht benötigt</v>
+      </c>
+      <c r="K29" t="str">
+        <f>IFERROR(VLOOKUP($A29,Parts!$A$2:$S$200,10,FALSE),"")</f>
+        <v>https://www.reichelt.de/de/de/shop/produkt/widerstand_metallschicht_150_ohm_0207_250_mw_0_1_-237515</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" ht="15" customHeight="1">
+      <c r="A30" t="s">
+        <v>304</v>
+      </c>
+      <c r="B30" s="39" t="str">
+        <f>IFERROR(VLOOKUP($A30,Parts!$A$2:$S$200,3,FALSE),"")</f>
+        <v>Schnelle Schaltdiode 1N4148W</v>
+      </c>
+      <c r="C30" t="str">
+        <f>IFERROR(VLOOKUP($A30,Parts!$A$2:$S$200,8,FALSE),"")</f>
+        <v>reichelt</v>
+      </c>
+      <c r="D30" t="str">
+        <f>IFERROR(VLOOKUP($A30,Parts!$A$2:$S$200,9,FALSE),"")</f>
+        <v>1N 4148W DIO</v>
+      </c>
+      <c r="E30" s="21">
+        <f>SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A30,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$5+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A30,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Optional")*$C$5,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A30,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"DNP")*$C$5,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A30,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$6+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A30,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Optional")*$C$6,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A30,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"DNP")*$C$6,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A30,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$7+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A30,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Optional")*$C$7,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A30,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"DNP")*$C$7,0)</f>
+        <v>4</v>
+      </c>
+      <c r="F30" s="21">
+        <f>IFERROR(VLOOKUP($A30,Parts!$A$2:$S$200,13,FALSE),"")</f>
+        <v>0</v>
+      </c>
+      <c r="G30" s="21">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="H30" s="38">
+        <f>IFERROR(VLOOKUP($A30,Parts!$A$2:$S$200,11,FALSE),0)</f>
+        <v>0.02</v>
+      </c>
+      <c r="I30" s="38">
+        <f t="shared" si="1"/>
+        <v>0.08</v>
+      </c>
+      <c r="J30" t="str">
+        <f t="shared" si="2"/>
+        <v>Reichelt bereit</v>
+      </c>
+      <c r="K30" t="str">
+        <f>IFERROR(VLOOKUP($A30,Parts!$A$2:$S$200,10,FALSE),"")</f>
+        <v>https://www.reichelt.de/de/de/shop/produkt/kleinsignal-schalt-diode_100_v_150_ma_sod-123-219382</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" ht="15" customHeight="1">
+      <c r="A31" t="s">
+        <v>311</v>
+      </c>
+      <c r="B31" s="39" t="str">
+        <f>IFERROR(VLOOKUP($A31,Parts!$A$2:$S$200,3,FALSE),"")</f>
+        <v>Schraubklemme 1x3, horizontal</v>
+      </c>
+      <c r="C31">
+        <f>IFERROR(VLOOKUP($A31,Parts!$A$2:$S$200,8,FALSE),"")</f>
+        <v>0</v>
+      </c>
+      <c r="D31">
+        <f>IFERROR(VLOOKUP($A31,Parts!$A$2:$S$200,9,FALSE),"")</f>
+        <v>0</v>
+      </c>
+      <c r="E31" s="21">
+        <f>SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A31,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$5+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A31,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Optional")*$C$5,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A31,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"DNP")*$C$5,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A31,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$6+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A31,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Optional")*$C$6,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A31,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"DNP")*$C$6,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A31,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$7+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A31,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Optional")*$C$7,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A31,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"DNP")*$C$7,0)</f>
+        <v>4</v>
+      </c>
+      <c r="F31" s="21">
+        <f>IFERROR(VLOOKUP($A31,Parts!$A$2:$S$200,13,FALSE),"")</f>
+        <v>0</v>
+      </c>
+      <c r="G31" s="21">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="H31" s="38">
+        <f>IFERROR(VLOOKUP($A31,Parts!$A$2:$S$200,11,FALSE),0)</f>
+        <v>0</v>
+      </c>
+      <c r="I31" s="38">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J31" t="str">
+        <f t="shared" si="2"/>
+        <v>Anderer Lieferant</v>
+      </c>
+      <c r="K31">
+        <f>IFERROR(VLOOKUP($A31,Parts!$A$2:$S$200,10,FALSE),"")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" ht="15" customHeight="1">
+      <c r="A32" t="s">
+        <v>318</v>
+      </c>
+      <c r="B32" s="39" t="str">
+        <f>IFERROR(VLOOKUP($A32,Parts!$A$2:$S$200,3,FALSE),"")</f>
+        <v>NPN-Transistor BC817</v>
+      </c>
+      <c r="C32" t="str">
+        <f>IFERROR(VLOOKUP($A32,Parts!$A$2:$S$200,8,FALSE),"")</f>
+        <v>reichelt</v>
+      </c>
+      <c r="D32" t="str">
+        <f>IFERROR(VLOOKUP($A32,Parts!$A$2:$S$200,9,FALSE),"")</f>
+        <v>BC 817-25 DIO</v>
+      </c>
+      <c r="E32" s="21">
+        <f>SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A32,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$5+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A32,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Optional")*$C$5,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A32,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"DNP")*$C$5,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A32,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$6+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A32,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Optional")*$C$6,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A32,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"DNP")*$C$6,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A32,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$7+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A32,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Optional")*$C$7,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A32,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"DNP")*$C$7,0)</f>
+        <v>4</v>
+      </c>
+      <c r="F32" s="21">
+        <f>IFERROR(VLOOKUP($A32,Parts!$A$2:$S$200,13,FALSE),"")</f>
+        <v>0</v>
+      </c>
+      <c r="G32" s="21">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="H32" s="38">
+        <f>IFERROR(VLOOKUP($A32,Parts!$A$2:$S$200,11,FALSE),0)</f>
+        <v>0.02</v>
+      </c>
+      <c r="I32" s="38">
+        <f t="shared" si="1"/>
+        <v>0.08</v>
+      </c>
+      <c r="J32" t="str">
+        <f t="shared" si="2"/>
+        <v>Reichelt bereit</v>
+      </c>
+      <c r="K32" t="str">
+        <f>IFERROR(VLOOKUP($A32,Parts!$A$2:$S$200,10,FALSE),"")</f>
+        <v>https://www.reichelt.de/de/de/shop/produkt/bipolartransistor_npn_45v_0_5a_0_25w_sot-23-219186</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" ht="15" customHeight="1">
+      <c r="A33" t="s">
+        <v>326</v>
+      </c>
+      <c r="B33" s="39" t="str">
+        <f>IFERROR(VLOOKUP($A33,Parts!$A$2:$S$200,3,FALSE),"")</f>
+        <v>Widerstand 1 kΩ SMD</v>
+      </c>
+      <c r="C33" t="str">
+        <f>IFERROR(VLOOKUP($A33,Parts!$A$2:$S$200,8,FALSE),"")</f>
+        <v>reichelt</v>
+      </c>
+      <c r="D33" t="str">
+        <f>IFERROR(VLOOKUP($A33,Parts!$A$2:$S$200,9,FALSE),"")</f>
+        <v>VIS CRCW12061K0</v>
+      </c>
+      <c r="E33" s="21">
+        <f>SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A33,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$5+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A33,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Optional")*$C$5,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A33,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"DNP")*$C$5,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A33,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$6+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A33,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Optional")*$C$6,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A33,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"DNP")*$C$6,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A33,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$7+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A33,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Optional")*$C$7,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A33,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"DNP")*$C$7,0)</f>
+        <v>4</v>
+      </c>
+      <c r="F33" s="21">
+        <f>IFERROR(VLOOKUP($A33,Parts!$A$2:$S$200,13,FALSE),"")</f>
+        <v>0</v>
+      </c>
+      <c r="G33" s="21">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="H33" s="38">
+        <f>IFERROR(VLOOKUP($A33,Parts!$A$2:$S$200,11,FALSE),0)</f>
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="I33" s="38">
+        <f t="shared" si="1"/>
+        <v>0.56000000000000005</v>
+      </c>
+      <c r="J33" t="str">
+        <f t="shared" si="2"/>
+        <v>Reichelt bereit</v>
+      </c>
+      <c r="K33" t="str">
+        <f>IFERROR(VLOOKUP($A33,Parts!$A$2:$S$200,10,FALSE),"")</f>
+        <v>https://www.reichelt.de/de/de/shop/produkt/smd-widerstand_1206_1_0_kohm_250_mw_1_-238107?PROVID=2788&amp;gad_source=1&amp;gad_campaignid=1622074784&amp;gbraid=0AAAAADwnxtbRDWe6ThqPkANhw_ak4jWBw&amp;gclid=Cj0KCQjwnbrUBhDOARIsAKKhPpdctdiA6tqULvTn2sTUS6FqmJC1_J6HoVQmYOjjMGhSPlfi9dK4bSQaAmesEALw_wcB</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" ht="15" customHeight="1">
+      <c r="A34" t="s">
+        <v>443</v>
+      </c>
+      <c r="B34" s="39" t="str">
+        <f>IFERROR(VLOOKUP($A34,Parts!$A$2:$S$200,3,FALSE),"")</f>
+        <v>Buchsenleiste 2x7, 2,54 mm, vertikal</v>
+      </c>
+      <c r="C34" t="str">
+        <f>IFERROR(VLOOKUP($A34,Parts!$A$2:$S$200,8,FALSE),"")</f>
+        <v>DigiKey</v>
+      </c>
+      <c r="D34" t="str">
+        <f>IFERROR(VLOOKUP($A34,Parts!$A$2:$S$200,9,FALSE),"")</f>
+        <v>732-61301421821-ND</v>
+      </c>
+      <c r="E34" s="21">
+        <f>SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A34,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$5+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A34,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Optional")*$C$5,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A34,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"DNP")*$C$5,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A34,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$6+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A34,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Optional")*$C$6,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A34,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"DNP")*$C$6,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A34,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$7+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A34,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Optional")*$C$7,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A34,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"DNP")*$C$7,0)</f>
+        <v>2</v>
+      </c>
+      <c r="F34" s="21">
+        <f>IFERROR(VLOOKUP($A34,Parts!$A$2:$S$200,13,FALSE),"")</f>
+        <v>0</v>
+      </c>
+      <c r="G34" s="21">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="H34" s="38">
+        <f>IFERROR(VLOOKUP($A34,Parts!$A$2:$S$200,11,FALSE),0)</f>
+        <v>0.56000000000000005</v>
+      </c>
+      <c r="I34" s="38">
+        <f t="shared" si="1"/>
+        <v>1.1200000000000001</v>
+      </c>
+      <c r="J34" t="str">
+        <f t="shared" si="2"/>
+        <v>Anderer Lieferant</v>
+      </c>
+      <c r="K34" t="str">
+        <f>IFERROR(VLOOKUP($A34,Parts!$A$2:$S$200,10,FALSE),"")</f>
+        <v>https://www.digikey.de/de/products/detail/w%C3%BCrth-elektronik/61301421821/16608590</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" ht="15" customHeight="1">
+      <c r="A35" t="s">
+        <v>457</v>
+      </c>
+      <c r="B35" s="39" t="str">
+        <f>IFERROR(VLOOKUP($A35,Parts!$A$2:$S$200,3,FALSE),"")</f>
+        <v>Schottky-Diode SS14, SMA</v>
+      </c>
+      <c r="C35" t="str">
+        <f>IFERROR(VLOOKUP($A35,Parts!$A$2:$S$200,8,FALSE),"")</f>
+        <v>reichelt</v>
+      </c>
+      <c r="D35" t="str">
+        <f>IFERROR(VLOOKUP($A35,Parts!$A$2:$S$200,9,FALSE),"")</f>
+        <v>SS 14 VIS</v>
+      </c>
+      <c r="E35" s="21">
+        <f>SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A35,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$5+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A35,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Optional")*$C$5,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A35,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"DNP")*$C$5,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A35,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$6+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A35,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Optional")*$C$6,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A35,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"DNP")*$C$6,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A35,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$7+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A35,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Optional")*$C$7,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A35,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"DNP")*$C$7,0)</f>
+        <v>2</v>
+      </c>
+      <c r="F35" s="21">
+        <f>IFERROR(VLOOKUP($A35,Parts!$A$2:$S$200,13,FALSE),"")</f>
+        <v>0</v>
+      </c>
+      <c r="G35" s="21">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="H35" s="38">
+        <f>IFERROR(VLOOKUP($A35,Parts!$A$2:$S$200,11,FALSE),0)</f>
+        <v>0.18</v>
+      </c>
+      <c r="I35" s="38">
+        <f t="shared" si="1"/>
+        <v>0.36</v>
+      </c>
+      <c r="J35" t="str">
+        <f t="shared" si="2"/>
+        <v>Reichelt bereit</v>
+      </c>
+      <c r="K35" t="str">
+        <f>IFERROR(VLOOKUP($A35,Parts!$A$2:$S$200,10,FALSE),"")</f>
+        <v>https://www.reichelt.de/de/de/shop/produkt/schottkydiode_40_v_1_a_do-214ac-219612</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" ht="15" customHeight="1">
+      <c r="A36" t="s">
+        <v>466</v>
+      </c>
+      <c r="B36" s="39" t="str">
+        <f>IFERROR(VLOOKUP($A36,Parts!$A$2:$S$200,3,FALSE),"")</f>
+        <v>Elektrolytkondensator 10 µF SMD</v>
+      </c>
+      <c r="C36" t="str">
+        <f>IFERROR(VLOOKUP($A36,Parts!$A$2:$S$200,8,FALSE),"")</f>
+        <v>reichelt</v>
+      </c>
+      <c r="D36" t="str">
+        <f>IFERROR(VLOOKUP($A36,Parts!$A$2:$S$200,9,FALSE),"")</f>
+        <v>S-V 10U 25</v>
+      </c>
+      <c r="E36" s="21">
+        <f>SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A36,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$5+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A36,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Optional")*$C$5,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A36,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"DNP")*$C$5,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A36,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$6+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A36,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Optional")*$C$6,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A36,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"DNP")*$C$6,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A36,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$7+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A36,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Optional")*$C$7,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A36,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"DNP")*$C$7,0)</f>
+        <v>1</v>
+      </c>
+      <c r="F36" s="21">
+        <f>IFERROR(VLOOKUP($A36,Parts!$A$2:$S$200,13,FALSE),"")</f>
+        <v>0</v>
+      </c>
+      <c r="G36" s="21">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="H36" s="38">
+        <f>IFERROR(VLOOKUP($A36,Parts!$A$2:$S$200,11,FALSE),0)</f>
+        <v>0.18</v>
+      </c>
+      <c r="I36" s="38">
+        <f t="shared" si="1"/>
+        <v>0.18</v>
+      </c>
+      <c r="J36" t="str">
+        <f t="shared" si="2"/>
+        <v>Reichelt bereit</v>
+      </c>
+      <c r="K36" t="str">
+        <f>IFERROR(VLOOKUP($A36,Parts!$A$2:$S$200,10,FALSE),"")</f>
+        <v>https://www.reichelt.de/de/de/shop/produkt/smd-elko_10_f_-20_25_v_85_5_x_5_4_mm-228459</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" ht="15" customHeight="1">
+      <c r="A37" t="s">
+        <v>476</v>
+      </c>
+      <c r="B37" s="39" t="str">
+        <f>IFERROR(VLOOKUP($A37,Parts!$A$2:$S$200,3,FALSE),"")</f>
+        <v>EnvNode Mini PCB Rev 0.2</v>
+      </c>
+      <c r="C37" t="str">
+        <f>IFERROR(VLOOKUP($A37,Parts!$A$2:$S$200,8,FALSE),"")</f>
+        <v>JLCPCB</v>
+      </c>
+      <c r="D37">
+        <f>IFERROR(VLOOKUP($A37,Parts!$A$2:$S$200,9,FALSE),"")</f>
+        <v>0</v>
+      </c>
+      <c r="E37" s="21">
+        <f>SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A37,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$5+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A37,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Optional")*$C$5,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A37,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"DNP")*$C$5,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A37,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$6+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A37,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Optional")*$C$6,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A37,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"DNP")*$C$6,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A37,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$7+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A37,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Optional")*$C$7,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A37,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"DNP")*$C$7,0)</f>
+        <v>1</v>
+      </c>
+      <c r="F37" s="21">
+        <f>IFERROR(VLOOKUP($A37,Parts!$A$2:$S$200,13,FALSE),"")</f>
+        <v>0</v>
+      </c>
+      <c r="G37" s="21">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="H37" s="38">
+        <f>IFERROR(VLOOKUP($A37,Parts!$A$2:$S$200,11,FALSE),0)</f>
+        <v>0</v>
+      </c>
+      <c r="I37" s="38">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J37" t="str">
+        <f t="shared" si="2"/>
+        <v>Anderer Lieferant</v>
+      </c>
+      <c r="K37">
+        <f>IFERROR(VLOOKUP($A37,Parts!$A$2:$S$200,10,FALSE),"")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" ht="26.25" customHeight="1">
+      <c r="A38" t="s">
+        <v>491</v>
+      </c>
+      <c r="B38" s="39" t="str">
+        <f>IFERROR(VLOOKUP($A38,Parts!$A$2:$S$200,3,FALSE),"")</f>
+        <v>Stiftleiste 2x7, 2,54 mm, vertikal, Bottom-Mount</v>
+      </c>
+      <c r="C38" t="str">
+        <f>IFERROR(VLOOKUP($A38,Parts!$A$2:$S$200,8,FALSE),"")</f>
+        <v>Reichelt</v>
+      </c>
+      <c r="D38" t="str">
+        <f>IFERROR(VLOOKUP($A38,Parts!$A$2:$S$200,9,FALSE),"")</f>
+        <v>ECON SL14G2</v>
+      </c>
+      <c r="E38" s="21">
+        <f>SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A38,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$5+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A38,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Optional")*$C$5,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A38,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"DNP")*$C$5,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A38,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$6+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A38,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Optional")*$C$6,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A38,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"DNP")*$C$6,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A38,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$7+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A38,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Optional")*$C$7,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A38,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"DNP")*$C$7,0)</f>
+        <v>2</v>
+      </c>
+      <c r="F38" s="21">
+        <f>IFERROR(VLOOKUP($A38,Parts!$A$2:$S$200,13,FALSE),"")</f>
+        <v>0</v>
+      </c>
+      <c r="G38" s="21">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="H38" s="38">
+        <f>IFERROR(VLOOKUP($A38,Parts!$A$2:$S$200,11,FALSE),0)</f>
+        <v>0.3</v>
+      </c>
+      <c r="I38" s="38">
+        <f t="shared" si="1"/>
+        <v>0.6</v>
+      </c>
+      <c r="J38" t="str">
+        <f t="shared" si="2"/>
+        <v>Reichelt bereit</v>
+      </c>
+      <c r="K38" t="str">
+        <f>IFERROR(VLOOKUP($A38,Parts!$A$2:$S$200,10,FALSE),"")</f>
+        <v>https://www.reichelt.de/de/de/shop/produkt/stiftleiste_2_x_7_polig_gerade_rastermass_2_54_mm-404299</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" ht="15" customHeight="1">
+      <c r="A39" t="s">
+        <v>527</v>
+      </c>
+      <c r="B39" s="39" t="str">
+        <f>IFERROR(VLOOKUP($A39,Parts!$A$2:$S$200,3,FALSE),"")</f>
+        <v>LED SMD 1206, rot</v>
+      </c>
+      <c r="C39" t="str">
+        <f>IFERROR(VLOOKUP($A39,Parts!$A$2:$S$200,8,FALSE),"")</f>
+        <v>reichelt</v>
+      </c>
+      <c r="D39" t="str">
+        <f>IFERROR(VLOOKUP($A39,Parts!$A$2:$S$200,9,FALSE),"")</f>
+        <v>KBT KP-3216SURC</v>
+      </c>
+      <c r="E39" s="21">
+        <f>SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A39,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$5+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A39,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Optional")*$C$5,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A39,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"DNP")*$C$5,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A39,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$6+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A39,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Optional")*$C$6,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A39,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"DNP")*$C$6,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A39,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$7+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A39,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Optional")*$C$7,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A39,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"DNP")*$C$7,0)</f>
+        <v>4</v>
+      </c>
+      <c r="F39" s="21">
+        <f>IFERROR(VLOOKUP($A39,Parts!$A$2:$S$200,13,FALSE),"")</f>
+        <v>0</v>
+      </c>
+      <c r="G39" s="21">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="H39" s="38">
+        <f>IFERROR(VLOOKUP($A39,Parts!$A$2:$S$200,11,FALSE),0)</f>
+        <v>0.11</v>
+      </c>
+      <c r="I39" s="38">
+        <f t="shared" si="1"/>
+        <v>0.44</v>
+      </c>
+      <c r="J39" t="str">
+        <f t="shared" si="2"/>
+        <v>Reichelt bereit</v>
+      </c>
+      <c r="K39" t="str">
+        <f>IFERROR(VLOOKUP($A39,Parts!$A$2:$S$200,10,FALSE),"")</f>
+        <v>https://www.reichelt.de/de/de/shop/produkt/smd-led_1206_hyper-rot_250_mcd_645_nm_140_-231713</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" ht="15" customHeight="1">
+      <c r="A40" t="s">
+        <v>540</v>
+      </c>
+      <c r="B40" s="39" t="str">
+        <f>IFERROR(VLOOKUP($A40,Parts!$A$2:$S$200,3,FALSE),"")</f>
+        <v>Widerstand 1,5 kΩ SMD</v>
+      </c>
+      <c r="C40" t="str">
+        <f>IFERROR(VLOOKUP($A40,Parts!$A$2:$S$200,8,FALSE),"")</f>
+        <v>Reichelt</v>
+      </c>
+      <c r="D40" t="str">
+        <f>IFERROR(VLOOKUP($A40,Parts!$A$2:$S$200,9,FALSE),"")</f>
+        <v>VIS CRCW12061K5</v>
+      </c>
+      <c r="E40" s="21">
+        <f>SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A40,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$5+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A40,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Optional")*$C$5,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A40,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"DNP")*$C$5,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A40,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$6+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A40,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Optional")*$C$6,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A40,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"DNP")*$C$6,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A40,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$7+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A40,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Optional")*$C$7,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A40,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"DNP")*$C$7,0)</f>
+        <v>4</v>
+      </c>
+      <c r="F40" s="21">
+        <f>IFERROR(VLOOKUP($A40,Parts!$A$2:$S$200,13,FALSE),"")</f>
+        <v>0</v>
+      </c>
+      <c r="G40" s="21">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="H40" s="38">
+        <f>IFERROR(VLOOKUP($A40,Parts!$A$2:$S$200,11,FALSE),0)</f>
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="I40" s="38">
+        <f t="shared" si="1"/>
+        <v>0.56000000000000005</v>
+      </c>
+      <c r="J40" t="str">
+        <f t="shared" si="2"/>
+        <v>Reichelt bereit</v>
+      </c>
+      <c r="K40" t="str">
+        <f>IFERROR(VLOOKUP($A40,Parts!$A$2:$S$200,10,FALSE),"")</f>
+        <v>https://www.reichelt.de/de/de/shop/produkt/smd-widerstand_1206_1_5_kohm_250_mw_1_-238108</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" ht="15" customHeight="1">
+      <c r="A41" t="s">
+        <v>550</v>
+      </c>
+      <c r="B41" s="39" t="str">
+        <f>IFERROR(VLOOKUP($A41,Parts!$A$2:$S$200,3,FALSE),"")</f>
+        <v>DuoRelay FullSize PCB Rev 0.2</v>
+      </c>
+      <c r="C41" t="str">
+        <f>IFERROR(VLOOKUP($A41,Parts!$A$2:$S$200,8,FALSE),"")</f>
+        <v>JLCPCB</v>
+      </c>
+      <c r="D41">
+        <f>IFERROR(VLOOKUP($A41,Parts!$A$2:$S$200,9,FALSE),"")</f>
+        <v>0</v>
+      </c>
+      <c r="E41" s="21">
+        <f>SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A41,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$5+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A41,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Optional")*$C$5,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A41,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"DNP")*$C$5,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A41,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$6+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A41,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Optional")*$C$6,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A41,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"DNP")*$C$6,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A41,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$7+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A41,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Optional")*$C$7,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A41,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"DNP")*$C$7,0)</f>
+        <v>2</v>
+      </c>
+      <c r="F41" s="21">
+        <f>IFERROR(VLOOKUP($A41,Parts!$A$2:$S$200,13,FALSE),"")</f>
+        <v>0</v>
+      </c>
+      <c r="G41" s="21">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="H41" s="38">
+        <f>IFERROR(VLOOKUP($A41,Parts!$A$2:$S$200,11,FALSE),0)</f>
+        <v>0</v>
+      </c>
+      <c r="I41" s="38">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J41" t="str">
+        <f t="shared" si="2"/>
+        <v>Anderer Lieferant</v>
+      </c>
+      <c r="K41">
+        <f>IFERROR(VLOOKUP($A41,Parts!$A$2:$S$200,10,FALSE),"")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" ht="15" customHeight="1">
+      <c r="A42" t="s">
+        <v>554</v>
+      </c>
+      <c r="B42" s="39" t="str">
+        <f>IFERROR(VLOOKUP($A42,Parts!$A$2:$S$200,3,FALSE),"")</f>
+        <v>Keramikkondensator 4,7 µF SMD</v>
+      </c>
+      <c r="C42" t="str">
+        <f>IFERROR(VLOOKUP($A42,Parts!$A$2:$S$200,8,FALSE),"")</f>
+        <v>Reichelt</v>
+      </c>
+      <c r="D42" t="str">
+        <f>IFERROR(VLOOKUP($A42,Parts!$A$2:$S$200,9,FALSE),"")</f>
+        <v>CL31B475KAHNNNE</v>
+      </c>
+      <c r="E42" s="21">
+        <f>SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A42,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$5+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A42,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Optional")*$C$5,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A42,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"DNP")*$C$5,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A42,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$6+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A42,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Optional")*$C$6,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A42,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"DNP")*$C$6,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A42,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$7+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A42,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Optional")*$C$7,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A42,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"DNP")*$C$7,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F42" s="21">
+        <f>IFERROR(VLOOKUP($A42,Parts!$A$2:$S$200,13,FALSE),"")</f>
+        <v>0</v>
+      </c>
+      <c r="G42" s="21">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H42" s="38">
+        <f>IFERROR(VLOOKUP($A42,Parts!$A$2:$S$200,11,FALSE),0)</f>
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="I42" s="38">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J42" t="str">
+        <f t="shared" si="2"/>
+        <v>Nicht benötigt</v>
+      </c>
+      <c r="K42" t="str">
+        <f>IFERROR(VLOOKUP($A42,Parts!$A$2:$S$200,10,FALSE),"")</f>
+        <v>https://www.reichelt.de/de/de/shop/produkt/mlcc_1206_4_7uf_25v_x7r_-10_h1_6_mm-429143</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" ht="15" customHeight="1">
+      <c r="A43" t="s">
+        <v>563</v>
+      </c>
+      <c r="B43" s="39" t="str">
+        <f>IFERROR(VLOOKUP($A43,Parts!$A$2:$S$200,3,FALSE),"")</f>
+        <v>Keramikkondensator 4,7 µF SMD</v>
+      </c>
+      <c r="C43" t="str">
+        <f>IFERROR(VLOOKUP($A43,Parts!$A$2:$S$200,8,FALSE),"")</f>
+        <v>Reichelt</v>
+      </c>
+      <c r="D43" t="str">
+        <f>IFERROR(VLOOKUP($A43,Parts!$A$2:$S$200,9,FALSE),"")</f>
+        <v>CL32B475KBJVPNE</v>
+      </c>
+      <c r="E43" s="21">
+        <f>SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A43,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$5+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A43,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Optional")*$C$5,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A43,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"DNP")*$C$5,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A43,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$6+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A43,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Optional")*$C$6,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A43,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"DNP")*$C$6,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A43,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$7+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A43,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Optional")*$C$7,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A43,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"DNP")*$C$7,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F43" s="21">
+        <f>IFERROR(VLOOKUP($A43,Parts!$A$2:$S$200,13,FALSE),"")</f>
+        <v>0</v>
+      </c>
+      <c r="G43" s="21">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H43" s="38">
+        <f>IFERROR(VLOOKUP($A43,Parts!$A$2:$S$200,11,FALSE),0)</f>
+        <v>1.19</v>
+      </c>
+      <c r="I43" s="38">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J43" t="str">
+        <f t="shared" si="2"/>
+        <v>Nicht benötigt</v>
+      </c>
+      <c r="K43" t="str">
+        <f>IFERROR(VLOOKUP($A43,Parts!$A$2:$S$200,10,FALSE),"")</f>
+        <v>https://www.reichelt.de/de/de/shop/produkt/mlcc_1210_4_7_f_50v_x7r_-10_-438066</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" ht="15" customHeight="1">
+      <c r="A44" t="s">
+        <v>571</v>
+      </c>
+      <c r="B44" s="39" t="str">
+        <f>IFERROR(VLOOKUP($A44,Parts!$A$2:$S$200,3,FALSE),"")</f>
+        <v>Schottky-Diode SMD</v>
+      </c>
+      <c r="C44">
+        <f>IFERROR(VLOOKUP($A44,Parts!$A$2:$S$200,8,FALSE),"")</f>
+        <v>0</v>
+      </c>
+      <c r="D44">
+        <f>IFERROR(VLOOKUP($A44,Parts!$A$2:$S$200,9,FALSE),"")</f>
+        <v>0</v>
+      </c>
+      <c r="E44" s="21">
+        <f>SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A44,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$5+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A44,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Optional")*$C$5,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A44,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"DNP")*$C$5,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A44,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$6+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A44,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Optional")*$C$6,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A44,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"DNP")*$C$6,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A44,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$7+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A44,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Optional")*$C$7,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A44,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"DNP")*$C$7,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F44" s="21">
+        <f>IFERROR(VLOOKUP($A44,Parts!$A$2:$S$200,13,FALSE),"")</f>
+        <v>0</v>
+      </c>
+      <c r="G44" s="21">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H44" s="38">
+        <f>IFERROR(VLOOKUP($A44,Parts!$A$2:$S$200,11,FALSE),0)</f>
+        <v>0</v>
+      </c>
+      <c r="I44" s="38">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J44" t="str">
+        <f t="shared" si="2"/>
+        <v>Nicht benötigt</v>
+      </c>
+      <c r="K44">
+        <f>IFERROR(VLOOKUP($A44,Parts!$A$2:$S$200,10,FALSE),"")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" ht="15" customHeight="1">
+      <c r="A45" t="s">
+        <v>578</v>
+      </c>
+      <c r="B45" s="39" t="str">
+        <f>IFERROR(VLOOKUP($A45,Parts!$A$2:$S$200,3,FALSE),"")</f>
+        <v>Leistungsinduktivität 0,68 µH</v>
+      </c>
+      <c r="C45" t="str">
+        <f>IFERROR(VLOOKUP($A45,Parts!$A$2:$S$200,8,FALSE),"")</f>
+        <v>Mouser</v>
+      </c>
+      <c r="D45" t="str">
+        <f>IFERROR(VLOOKUP($A45,Parts!$A$2:$S$200,9,FALSE),"")</f>
+        <v>710-744383560068</v>
+      </c>
+      <c r="E45" s="21">
+        <f>SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A45,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$5+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A45,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Optional")*$C$5,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A45,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"DNP")*$C$5,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A45,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$6+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A45,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Optional")*$C$6,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A45,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"DNP")*$C$6,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A45,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$7+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A45,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Optional")*$C$7,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A45,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"DNP")*$C$7,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F45" s="21">
+        <f>IFERROR(VLOOKUP($A45,Parts!$A$2:$S$200,13,FALSE),"")</f>
+        <v>0</v>
+      </c>
+      <c r="G45" s="21">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H45" s="38">
+        <f>IFERROR(VLOOKUP($A45,Parts!$A$2:$S$200,11,FALSE),0)</f>
+        <v>1.66</v>
+      </c>
+      <c r="I45" s="38">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J45" t="str">
+        <f t="shared" si="2"/>
+        <v>Nicht benötigt</v>
+      </c>
+      <c r="K45" t="str">
+        <f>IFERROR(VLOOKUP($A45,Parts!$A$2:$S$200,10,FALSE),"")</f>
+        <v>https://eu.mouser.com/en/ProductDetail/Wurth-Elektronik/744383560068</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" ht="15" customHeight="1">
+      <c r="A46" t="s">
+        <v>591</v>
+      </c>
+      <c r="B46" s="39" t="str">
+        <f>IFERROR(VLOOKUP($A46,Parts!$A$2:$S$200,3,FALSE),"")</f>
+        <v>Widerstand 1 MΩ SMD</v>
+      </c>
+      <c r="C46" t="str">
+        <f>IFERROR(VLOOKUP($A46,Parts!$A$2:$S$200,8,FALSE),"")</f>
+        <v>Reichelt</v>
+      </c>
+      <c r="D46" t="str">
+        <f>IFERROR(VLOOKUP($A46,Parts!$A$2:$S$200,9,FALSE),"")</f>
+        <v>VIS CRCW12061M0</v>
+      </c>
+      <c r="E46" s="21">
+        <f>SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A46,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$5+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A46,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Optional")*$C$5,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A46,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"DNP")*$C$5,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A46,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$6+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A46,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Optional")*$C$6,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A46,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"DNP")*$C$6,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A46,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$7+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A46,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Optional")*$C$7,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A46,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"DNP")*$C$7,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F46" s="21">
+        <f>IFERROR(VLOOKUP($A46,Parts!$A$2:$S$200,13,FALSE),"")</f>
+        <v>0</v>
+      </c>
+      <c r="G46" s="21">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H46" s="38">
+        <f>IFERROR(VLOOKUP($A46,Parts!$A$2:$S$200,11,FALSE),0)</f>
+        <v>0.18</v>
+      </c>
+      <c r="I46" s="38">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J46" t="str">
+        <f t="shared" si="2"/>
+        <v>Nicht benötigt</v>
+      </c>
+      <c r="K46" t="str">
+        <f>IFERROR(VLOOKUP($A46,Parts!$A$2:$S$200,10,FALSE),"")</f>
+        <v>https://www.reichelt.de/de/de/shop/produkt/smd-widerstand_1206_1_0_mohm_250_mw_1_-238109</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" ht="15" customHeight="1">
+      <c r="A47" t="s">
+        <v>600</v>
+      </c>
+      <c r="B47" s="39" t="str">
+        <f>IFERROR(VLOOKUP($A47,Parts!$A$2:$S$200,3,FALSE),"")</f>
+        <v>Widerstand 71,5 kΩ SMD</v>
+      </c>
+      <c r="C47" t="str">
+        <f>IFERROR(VLOOKUP($A47,Parts!$A$2:$S$200,8,FALSE),"")</f>
+        <v>DigiKey</v>
+      </c>
+      <c r="D47">
+        <f>IFERROR(VLOOKUP($A47,Parts!$A$2:$S$200,9,FALSE),"")</f>
+        <v>0</v>
+      </c>
+      <c r="E47" s="21">
+        <f>SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A47,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$5+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A47,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Optional")*$C$5,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A47,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"DNP")*$C$5,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A47,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$6+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A47,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Optional")*$C$6,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A47,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"DNP")*$C$6,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A47,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$7+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A47,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Optional")*$C$7,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A47,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"DNP")*$C$7,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F47" s="21">
+        <f>IFERROR(VLOOKUP($A47,Parts!$A$2:$S$200,13,FALSE),"")</f>
+        <v>0</v>
+      </c>
+      <c r="G47" s="21">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H47" s="38">
+        <f>IFERROR(VLOOKUP($A47,Parts!$A$2:$S$200,11,FALSE),0)</f>
+        <v>0.09</v>
+      </c>
+      <c r="I47" s="38">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J47" t="str">
+        <f t="shared" si="2"/>
+        <v>Nicht benötigt</v>
+      </c>
+      <c r="K47" t="str">
+        <f>IFERROR(VLOOKUP($A47,Parts!$A$2:$S$200,10,FALSE),"")</f>
+        <v>https://www.digikey.de/de/products/filter/chipwiderstand-oberfl%C3%A4chenmontage/71-5-kohms/52</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" ht="15" customHeight="1">
+      <c r="A48" t="s">
+        <v>609</v>
+      </c>
+      <c r="B48" s="39" t="str">
+        <f>IFERROR(VLOOKUP($A48,Parts!$A$2:$S$200,3,FALSE),"")</f>
+        <v>Widerstand 220 kΩ SMD</v>
+      </c>
+      <c r="C48" t="str">
+        <f>IFERROR(VLOOKUP($A48,Parts!$A$2:$S$200,8,FALSE),"")</f>
+        <v>TME</v>
+      </c>
+      <c r="D48" t="str">
+        <f>IFERROR(VLOOKUP($A48,Parts!$A$2:$S$200,9,FALSE),"")</f>
+        <v>WR12X2203FTL</v>
+      </c>
+      <c r="E48" s="21">
+        <f>SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A48,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$5+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A48,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Optional")*$C$5,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A48,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"DNP")*$C$5,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A48,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$6+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A48,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Optional")*$C$6,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A48,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"DNP")*$C$6,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A48,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$7+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A48,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Optional")*$C$7,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A48,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"DNP")*$C$7,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F48" s="21">
+        <f>IFERROR(VLOOKUP($A48,Parts!$A$2:$S$200,13,FALSE),"")</f>
+        <v>0</v>
+      </c>
+      <c r="G48" s="21">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H48" s="38">
+        <f>IFERROR(VLOOKUP($A48,Parts!$A$2:$S$200,11,FALSE),0)</f>
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="I48" s="38">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J48" t="str">
+        <f t="shared" si="2"/>
+        <v>Nicht benötigt</v>
+      </c>
+      <c r="K48" t="str">
+        <f>IFERROR(VLOOKUP($A48,Parts!$A$2:$S$200,10,FALSE),"")</f>
+        <v>https://www.tme.eu/de/details/wr12x2203ftl/smd-widerstaende/walsin/</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" ht="15" customHeight="1">
+      <c r="A49" t="s">
+        <v>620</v>
+      </c>
+      <c r="B49" s="39" t="str">
+        <f>IFERROR(VLOOKUP($A49,Parts!$A$2:$S$200,3,FALSE),"")</f>
+        <v>Schiebeschalter DPDT</v>
+      </c>
+      <c r="C49" t="str">
+        <f>IFERROR(VLOOKUP($A49,Parts!$A$2:$S$200,8,FALSE),"")</f>
+        <v>Mouser</v>
+      </c>
+      <c r="D49" t="str">
+        <f>IFERROR(VLOOKUP($A49,Parts!$A$2:$S$200,9,FALSE),"")</f>
+        <v>611-OS202011MS2QS1</v>
+      </c>
+      <c r="E49" s="21">
+        <f>SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A49,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$5+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A49,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Optional")*$C$5,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A49,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"DNP")*$C$5,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A49,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$6+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A49,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Optional")*$C$6,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A49,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"DNP")*$C$6,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A49,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$7+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A49,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Optional")*$C$7,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A49,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"DNP")*$C$7,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F49" s="21">
+        <f>IFERROR(VLOOKUP($A49,Parts!$A$2:$S$200,13,FALSE),"")</f>
+        <v>0</v>
+      </c>
+      <c r="G49" s="21">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H49" s="38">
+        <f>IFERROR(VLOOKUP($A49,Parts!$A$2:$S$200,11,FALSE),0)</f>
+        <v>0.92</v>
+      </c>
+      <c r="I49" s="38">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J49" t="str">
+        <f t="shared" si="2"/>
+        <v>Nicht benötigt</v>
+      </c>
+      <c r="K49" t="str">
+        <f>IFERROR(VLOOKUP($A49,Parts!$A$2:$S$200,10,FALSE),"")</f>
+        <v>https://www.mouser.de/de/c/electromechanical/switches/slide-switches/?q=OS202011MS2QS1</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" ht="15" customHeight="1">
+      <c r="A50" t="s">
+        <v>632</v>
+      </c>
+      <c r="B50" s="39" t="str">
+        <f>IFERROR(VLOOKUP($A50,Parts!$A$2:$S$200,3,FALSE),"")</f>
+        <v>Boost-Regler LT8330</v>
+      </c>
+      <c r="C50" t="str">
+        <f>IFERROR(VLOOKUP($A50,Parts!$A$2:$S$200,8,FALSE),"")</f>
+        <v>Mouser</v>
+      </c>
+      <c r="D50" t="str">
+        <f>IFERROR(VLOOKUP($A50,Parts!$A$2:$S$200,9,FALSE),"")</f>
+        <v>584-LT8330ES6#TRMPBF</v>
+      </c>
+      <c r="E50" s="21">
+        <f>SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A50,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$5+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A50,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Optional")*$C$5,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A50,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"DNP")*$C$5,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A50,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$6+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A50,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Optional")*$C$6,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A50,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"DNP")*$C$6,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A50,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$7+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A50,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Optional")*$C$7,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A50,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"DNP")*$C$7,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F50" s="21">
+        <f>IFERROR(VLOOKUP($A50,Parts!$A$2:$S$200,13,FALSE),"")</f>
+        <v>0</v>
+      </c>
+      <c r="G50" s="21">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H50" s="38">
+        <f>IFERROR(VLOOKUP($A50,Parts!$A$2:$S$200,11,FALSE),0)</f>
+        <v>7.11</v>
+      </c>
+      <c r="I50" s="38">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J50" t="str">
+        <f t="shared" si="2"/>
+        <v>Nicht benötigt</v>
+      </c>
+      <c r="K50" t="str">
+        <f>IFERROR(VLOOKUP($A50,Parts!$A$2:$S$200,10,FALSE),"")</f>
+        <v>https://www.mouser.de/ProductDetail/Analog-Devices/LT8330ES6TRMPBF</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" ht="15" customHeight="1">
+      <c r="A51" t="s">
+        <v>643</v>
+      </c>
+      <c r="B51" s="39" t="str">
+        <f>IFERROR(VLOOKUP($A51,Parts!$A$2:$S$200,3,FALSE),"")</f>
+        <v>AnalogHydroPressure FullSize PCB Rev 0.2</v>
+      </c>
+      <c r="C51" t="str">
+        <f>IFERROR(VLOOKUP($A51,Parts!$A$2:$S$200,8,FALSE),"")</f>
+        <v>JLCPCB</v>
+      </c>
+      <c r="D51">
+        <f>IFERROR(VLOOKUP($A51,Parts!$A$2:$S$200,9,FALSE),"")</f>
+        <v>0</v>
+      </c>
+      <c r="E51" s="21">
+        <f>SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A51,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$5+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A51,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"Optional")*$C$5,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A51,Kit_BOM!$A$2:$A$65,$A$5,Kit_BOM!$G$2:$G$65,"DNP")*$C$5,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A51,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$6+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A51,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"Optional")*$C$6,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A51,Kit_BOM!$A$2:$A$65,$A$6,Kit_BOM!$G$2:$G$65,"DNP")*$C$6,0)+SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A51,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Bestücken")*$C$7+IF($F$5="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A51,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"Optional")*$C$7,0)+IF($F$6="Ja",SUMIFS(Kit_BOM!$F$2:$F$65,Kit_BOM!$E$2:$E$65,$A51,Kit_BOM!$A$2:$A$65,$A$7,Kit_BOM!$G$2:$G$65,"DNP")*$C$7,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F51" s="21">
+        <f>IFERROR(VLOOKUP($A51,Parts!$A$2:$S$200,13,FALSE),"")</f>
+        <v>0</v>
+      </c>
+      <c r="G51" s="21">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H51" s="38">
+        <f>IFERROR(VLOOKUP($A51,Parts!$A$2:$S$200,11,FALSE),0)</f>
+        <v>0</v>
+      </c>
+      <c r="I51" s="38">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J51" t="str">
+        <f t="shared" si="2"/>
+        <v>Nicht benötigt</v>
+      </c>
+      <c r="K51">
+        <f>IFERROR(VLOOKUP($A51,Parts!$A$2:$S$200,10,FALSE),"")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11">
+      <c r="A52" t="s">
+        <v>703</v>
+      </c>
+      <c r="I52" s="38">
+        <f>SUBTOTAL(109,OrderListTable[Bestellwert_EUR])</f>
+        <v>59.989999999999995</v>
+      </c>
+      <c r="K52">
+        <f>SUBTOTAL(103,OrderListTable[URL])</f>
+        <v>38</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="F8:K9"/>
+  </mergeCells>
+  <conditionalFormatting sqref="A14:K51">
+    <cfRule type="expression" dxfId="3" priority="4">
+      <formula>$E14=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J14:J51">
+    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="Reichelt bereit"/>
+    <cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Anderer Lieferant"/>
+    <cfRule type="containsText" dxfId="0" priority="3" operator="containsText" text="Supplier-PN fehlt"/>
+  </conditionalFormatting>
+  <dataValidations count="2">
+    <dataValidation type="whole" sqref="C5:C7" xr:uid="{00000000-0002-0000-0300-000000000000}">
+      <formula1>0</formula1>
+      <formula2>999</formula2>
+    </dataValidation>
+    <dataValidation type="list" sqref="F5:F6" xr:uid="{00000000-0002-0000-0300-000001000000}">
+      <formula1>"Nein,Ja"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(hardware): use SMD JST-PH on ORing power module
</commit_message>
<xml_diff>
--- a/hardware/EnvNode_Parts.xlsx
+++ b/hardware/EnvNode_Parts.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parts" sheetId="1" r:id="R7d5abe6f6c9c4c5e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kits" sheetId="2" r:id="R38154a1266ca410f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kit_BOM" sheetId="3" r:id="R16051e1b68c3410e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Order_List" sheetId="4" r:id="Rd03ca53372c14e64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stock" sheetId="6" r:id="R19389e9ed13e426d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Etiketten_Druck" sheetId="7" r:id="R96fb711129624da2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Part_Suppliers" sheetId="8" r:id="R2f82390d3a024244"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suppliers" sheetId="9" r:id="R6d2c2687664d48dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Part_Alternatives" sheetId="10" r:id="R14e4549456124a4d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parts" sheetId="1" r:id="R671ba58f9cc84284"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kits" sheetId="2" r:id="R6d126b74da924bb6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kit_BOM" sheetId="3" r:id="Re10a2a8f709e495e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Order_List" sheetId="4" r:id="R69c3bb1c44094f1d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stock" sheetId="6" r:id="R5ed8830f41cc41a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Etiketten_Druck" sheetId="7" r:id="R5aa922ca10134d4d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Part_Suppliers" sheetId="8" r:id="R415967df42c04cdd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suppliers" sheetId="9" r:id="Ra8efc125b0784878"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Part_Alternatives" sheetId="10" r:id="Rd121fb5a285b479a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4583,8 +4583,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="PartsTable" displayName="PartsTable" ref="A1:M119" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:M119"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="PartsTable" displayName="PartsTable" ref="A1:M120" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:M120"/>
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="Part_ID"/>
     <x:tableColumn id="2" name="Category"/>
@@ -4692,8 +4692,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="PartSuppliersTable" displayName="PartSuppliersTable" ref="A1:L119" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:L119"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="PartSuppliersTable" displayName="PartSuppliersTable" ref="A1:L120" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:L120"/>
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="Part_ID"/>
     <x:tableColumn id="2" name="Supplier"/>
@@ -9842,6 +9842,47 @@
         <x:v>ORING POWER MODUL PCB REV 0.1|PCB: DESIGNBLOCKS/ORING POWER/ORING POWER.KICAD_PCB</x:v>
       </x:c>
     </x:row>
+    <x:row r="120">
+      <x:c r="A120" t="str">
+        <x:v>ENP-00119</x:v>
+      </x:c>
+      <x:c r="B120" t="str">
+        <x:v>Steckverbinder</x:v>
+      </x:c>
+      <x:c r="C120" t="str">
+        <x:v>JST-PH Stiftleiste, 2-polig, vertikal, SMD</x:v>
+      </x:c>
+      <x:c r="D120" t="str">
+        <x:v>JST-PH, 2-polig, 2,00 mm, SMD</x:v>
+      </x:c>
+      <x:c r="E120" t="str">
+        <x:v>Connector_JST:JST_PH_B2B-PH-SM4-TB_1x02-1MP_P2.00mm_Vertical</x:v>
+      </x:c>
+      <x:c r="F120" t="str">
+        <x:v>JST</x:v>
+      </x:c>
+      <x:c r="G120" t="str">
+        <x:v>B2B-PH-SM4-TB</x:v>
+      </x:c>
+      <x:c r="H120" t="str">
+        <x:v>ORing Power Rev 0.1</x:v>
+      </x:c>
+      <x:c r="I120" t="str">
+        <x:v>J1</x:v>
+      </x:c>
+      <x:c r="J120" t="str">
+        <x:v>KiCad; JST PH Datenblatt; Reichelt, geprüft 2026-09-21</x:v>
+      </x:c>
+      <x:c r="K120" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="L120" t="str">
+        <x:v>Vertikale SMD-Ausführung mit zwei mechanischen Haltepads. Ersetzt ENP-00012 ausschließlich im ORing-Power-Modul.</x:v>
+      </x:c>
+      <x:c r="M120" t="str">
+        <x:v>B2B-PH-SM4-TB</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="Q2:Q54">
     <x:cfRule type="containsText" dxfId="11" priority="2" operator="containsText" text="Prüfen">
@@ -9861,11 +9902,11 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="R6fac5549e4454480"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="R5695e10d5add4472"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R81757a0c343d4c61"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a40d4efde834982"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10638,7 +10679,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra57768ce7f5a4922"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ee04d77cb594756"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15157,7 +15198,7 @@
         <x:v>J1</x:v>
       </x:c>
       <x:c r="E103" t="str">
-        <x:v>ENP-00012</x:v>
+        <x:v>ENP-00119</x:v>
       </x:c>
       <x:c r="F103" t="n">
         <x:v>1</x:v>
@@ -15169,19 +15210,19 @@
         <x:v>KiCad</x:v>
       </x:c>
       <x:c r="I103" t="str">
-        <x:v>JST-PH, 2-polig, 2,00 mm</x:v>
+        <x:v>JST-PH, 2-polig, 2,00 mm, SMD</x:v>
       </x:c>
       <x:c r="J103" t="str">
-        <x:v>Connector_JST:JST_PH_B2B-PH-K_1x02_P2.00mm_Vertical</x:v>
+        <x:v>Connector_JST:JST_PH_B2B-PH-SM4-TB_1x02-1MP_P2.00mm_Vertical</x:v>
       </x:c>
       <x:c r="K103" t="n">
-        <x:v>1.3</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="L103" t="n">
-        <x:v>1.3</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="M103" t="str">
-        <x:v>Alternativer 5-V-Eingang; liegt direkt parallel zu USB-VBUS.</x:v>
+        <x:v>Alternativer 5-V-Eingang; SMD-Ausführung B2B-PH-SM4-TB; liegt direkt parallel zu USB-VBUS.</x:v>
       </x:c>
       <x:c r="N103"/>
     </x:row>
@@ -15380,7 +15421,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c7c094aff194194"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red50ff5bdb5340c2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20140,7 +20181,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R24dda9cb03f943b8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8696efd0f997427b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -28946,7 +28987,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5bc9dcdf84184c51"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re29ccf0391a14338"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -33454,6 +33495,40 @@
         <x:v>ENP-00118|Ja</x:v>
       </x:c>
     </x:row>
+    <x:row r="120">
+      <x:c r="A120" t="str">
+        <x:v>ENP-00119</x:v>
+      </x:c>
+      <x:c r="B120" t="str">
+        <x:v>Reichelt</x:v>
+      </x:c>
+      <x:c r="C120" t="str">
+        <x:v>JST PH2P SMD</x:v>
+      </x:c>
+      <x:c r="D120" t="str">
+        <x:v>https://www.reichelt.de/de/de/shop/produkt/jst_-_stiftleiste_rm_2_mm_1x2_polig_gerade_-_ph-190546</x:v>
+      </x:c>
+      <x:c r="E120"/>
+      <x:c r="F120" t="str">
+        <x:v>Stk</x:v>
+      </x:c>
+      <x:c r="G120"/>
+      <x:c r="H120" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="I120" t="n">
+        <x:v>46286</x:v>
+      </x:c>
+      <x:c r="J120" t="str">
+        <x:v>SMD-Ausführung B2B-PH-SM4-TB; Preis vor Bestellung prüfen.</x:v>
+      </x:c>
+      <x:c r="K120" t="str">
+        <x:v>ENP-00119|Reichelt</x:v>
+      </x:c>
+      <x:c r="L120" t="str">
+        <x:v>ENP-00119|Ja</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="H2:H102">
@@ -33462,12 +33537,12 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D113" r:id="R4a271ccb4daa41f6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D116" r:id="R307f630d9d9e44c8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D113" r:id="Rea9815ae5c67400e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D116" r:id="Rbacb44e1252047d4"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R33938bb9af644938"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0392fc22d5ce4555"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -33576,7 +33651,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb539bbaf92a44223"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R53d6a7e5ee914e40"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -33759,7 +33834,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3663cee1a43e4449"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb75a31fc8d345e8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>